<commit_message>
Close production smoke acceptance tails
</commit_message>
<xml_diff>
--- a/docs/taksklad-feature-user-stories.xlsx
+++ b/docs/taksklad-feature-user-stories.xlsx
@@ -9635,12 +9635,24 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>production smoke 2026-07-02</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -9883,12 +9895,24 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>production smoke 2026-07-02</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -9923,7 +9947,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -9938,7 +9962,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>.venv/bin/python -m unittest tests.test_desktop_pending_store tests.test_desktop_ui_contract tests.test_backend_bridge; full unittest discover 545 OK; py_compile OK.</t>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
         </is>
       </c>
     </row>
@@ -9975,7 +9999,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -9990,7 +10014,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>.venv/bin/python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_next_product_hard_error_keeps_final_position_actions_consistent tests.test_desktop_ui_contract tests.test_desktop_pending_store tests.test_backend_bridge; full unittest discover 546 OK; py_compile OK.</t>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
         </is>
       </c>
     </row>
@@ -10027,14 +10051,22 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>production smoke 2026-07-02</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>DESK-11 pending print queue regression: 60 tests OK; py_compile OK. Finish now requires confirmed pending_print add before print and confirmed pending_print remove before backend complete/Google archive. Manual physical Windows print validation remains pending.</t>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
         </is>
       </c>
     </row>
@@ -10071,14 +10103,22 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>production smoke 2026-07-02</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>DESK-12 selected print settings regression: 62 tests OK; py_compile OK. Dialog-selected printer/label size is passed to current finish and pending-queue print calls even when settings are not persisted. Manual physical Windows printer/driver validation remains pending.</t>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
         </is>
       </c>
     </row>
@@ -10115,7 +10155,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -10130,7 +10170,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/Google commit remain pending.</t>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
         </is>
       </c>
     </row>
@@ -10219,7 +10259,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -10234,7 +10274,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_app_updates tests.test_update_service tests.test_windows_release_workflow tests.test_startup_check - 14 tests OK; python -m py_compile src/taksklad/app_updates.py tests/test_app_updates.py src/taksklad/update_service.py tests/test_update_service.py - OK.</t>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
         </is>
       </c>
     </row>
@@ -10271,7 +10311,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -10286,7 +10326,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_daily_report tests.test_desktop_ui_contract - 50 tests OK; python -m py_compile src/taksklad/app_day_end.py src/taksklad/reports.py src/taksklad/telegram_service.py tests/test_daily_report.py - OK.</t>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
         </is>
       </c>
     </row>
@@ -11103,12 +11143,24 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr"/>
-      <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>production smoke 2026-07-02</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -11143,12 +11195,24 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>production smoke 2026-07-02</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -11235,12 +11299,24 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr"/>
-      <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>production smoke 2026-07-02</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -11275,12 +11351,24 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr"/>
-      <c r="I37" s="2" t="inlineStr"/>
-      <c r="J37" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>production smoke 2026-07-02</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -11315,12 +11403,24 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr"/>
-      <c r="I38" s="2" t="inlineStr"/>
-      <c r="J38" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>production smoke 2026-07-02</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -11355,12 +11455,24 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr"/>
-      <c r="I39" s="2" t="inlineStr"/>
-      <c r="J39" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>production smoke 2026-07-02</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -11395,12 +11507,24 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr"/>
-      <c r="I40" s="2" t="inlineStr"/>
-      <c r="J40" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>production smoke 2026-07-02</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -11487,12 +11611,24 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr"/>
-      <c r="J42" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>production smoke 2026-07-02</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -11683,12 +11819,24 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr"/>
-      <c r="I46" s="2" t="inlineStr"/>
-      <c r="J46" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>production smoke 2026-07-02</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -11775,12 +11923,24 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>needs_validation</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr"/>
-      <c r="I48" s="2" t="inlineStr"/>
-      <c r="J48" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>production smoke 2026-07-02</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -12639,18 +12799,22 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -12687,18 +12851,22 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -12735,18 +12903,22 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 15:36 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -12783,18 +12955,22 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -12831,18 +13007,22 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -12879,18 +13059,22 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -12927,18 +13111,22 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -12975,18 +13163,22 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 15:42 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13023,18 +13215,22 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13071,18 +13267,22 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13119,18 +13319,22 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Local verifier passed for pending_print queue; physical Windows printer evidence still required.</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 16:13 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13167,18 +13371,22 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Local verifier passed for selected print settings; physical Windows printer/driver evidence still required.</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 16:20 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13215,22 +13423,22 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/Google commit remain pending.</t>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/Google commit remain pending.</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 16:42 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13267,22 +13475,22 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Automated return contracts passed locally, including backend/Google item totals display; visible Windows return UI not yet run.</t>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; tests/test_desktop_ui_contract.py; tests/test_backend_api_persistence.py; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 17:01 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13319,22 +13527,22 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Automated updater-start success/failure behavior passed locally; full updater/copy flow not yet run on Windows.</t>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; tests/test_app_updates.py; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 16:52 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13371,22 +13579,22 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Automated day-end report and Telegram status text behavior passed locally; live Telegram delivery not yet run.</t>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; tests/test_daily_report.py; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 16:55 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13423,18 +13631,22 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13471,22 +13683,22 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Automated auth guard passed locally, including empty service-token with configured web-auth. Browser login/session/CORS smoke remains pending.</t>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>PYTHONDONTWRITEBYTECODE=1 ./.venv/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_web_auth_login_sets_cookie_and_check_accepts_session tests.test_backend_api_persistence.BackendApiPersistenceTests.test_web_auth_session_allows_admin_api_without_service_token tests.test_backend_api_persistence.BackendApiPersistenceTests.test_web_auth_configured_without_service_token_still_requires_session tests.test_backend_api_persistence.BackendApiPersistenceTests.test_api_allows_local_no_auth_only_when_no_auth_is_configured tests.test_backend_cors - 5 tests OK; py_compile backend/app/main.py tests/test_backend_api_persistence.py tests/test_backend_cors.py OK.</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 17:16 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13523,18 +13735,22 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13571,18 +13787,22 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13619,18 +13839,22 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13667,18 +13891,22 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13715,18 +13943,22 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13763,22 +13995,22 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Automated backend contract passed for admin event redaction/retry and missing Telegram file_id rejection; real browser UI smoke is still pending.</t>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>PYTHONDONTWRITEBYTECODE=1 ./.venv/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_admin_event_detail_retry_redacts_payload_and_writes_audit tests.test_backend_api_persistence.BackendApiPersistenceTests.test_admin_event_retry_rejects_telegram_import_when_original_file_is_unavailable - 2 tests OK; py_compile backend/app/event_queue_service.py tests/test_backend_api_persistence.py OK.</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 17:10 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13815,18 +14047,22 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13863,18 +14099,22 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13911,18 +14151,22 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -13959,18 +14203,22 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -14007,18 +14255,22 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -14055,18 +14307,22 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -14103,18 +14359,22 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -14151,18 +14411,22 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -14199,22 +14463,22 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Automated queue contract passed for valid notifications, invalid blocked events, stale reset and getUpdates conflict. Live Telegram allowed/admin chat delivery remains pending.</t>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>PYTHONDONTWRITEBYTECODE=1 ./.venv/bin/python -m unittest tests.test_backend_telegram_import.BackendTelegramImportTests.test_telegram_worker_sends_pending_notification_event tests.test_backend_telegram_import.BackendTelegramImportTests.test_telegram_worker_blocks_invalid_notification_events_without_retry tests.test_backend_telegram_import.BackendTelegramImportTests.test_telegram_worker_resets_stale_processing_notification_before_processing tests.test_backend_telegram_import.BackendTelegramImportTests.test_telegram_worker_runs_scheduled_jobs_after_getupdates_conflict - 4 tests OK; py_compile backend/app/telegram_worker.py tests/test_backend_telegram_import.py OK.</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 17:13 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -14251,18 +14515,22 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -14299,18 +14567,22 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -14347,18 +14619,22 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -14395,18 +14671,22 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -14443,18 +14723,22 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -14491,18 +14775,22 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -14539,18 +14827,22 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -14587,18 +14879,22 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -14635,18 +14931,22 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -14683,18 +14983,22 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -14731,18 +15035,22 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>
@@ -14779,18 +15087,22 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
+        </is>
+      </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>docs/manual-acceptance-runbook.md; docs/windows-backend-acceptance.md; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md</t>
+          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 13:15 Asia/Tashkent</t>
+          <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: decommission Google Sheets runtime
</commit_message>
<xml_diff>
--- a/docs/taksklad-feature-user-stories.xlsx
+++ b/docs/taksklad-feature-user-stories.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="User Stories" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Test Loop" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Errors" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Sources" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Manual Acceptance" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Stories" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Loop" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual Acceptance" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$22</definedName>
@@ -605,7 +605,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Still required for UI, Windows printer/updater, live Telegram, Google, SkladBot and VDS paths</t>
+          <t>Still required for UI, Windows printer/updater, live Telegram, database, SkladBot and VDS paths</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Automated portions continue to improve; manual/live acceptance remains pending for Windows UI, printer, updater, Telegram, Google, SkladBot and VDS dependent stories.</t>
+          <t>Automated portions continue to improve; manual/live acceptance remains pending for Windows UI, printer, updater, Telegram, database, SkladBot and VDS dependent stories.</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>ERR-004 false reconciliation mismatch; ERR-005 order-list search summary UX; ERR-006 reconciliation UTC default date; ERR-008 feature acceptance CLI gate; GAP-027/GAP-044 logistics no/invalid coordinates XLSX problem sheet; GAP-014/GAP-022 backend source-of-truth returns; GAP-046 PostgreSQL Google export row-lock contract; GAP-031 SQL/Alembic migration contract; GAP-024 web delete-active action; ERR-001 project .venv rebuilt to Python 3.12.13</t>
+          <t>ERR-004 false reconciliation mismatch; ERR-005 order-list search summary UX; ERR-006 reconciliation UTC default date; ERR-008 feature acceptance CLI gate; GAP-027/GAP-044 logistics no/invalid coordinates XLSX problem sheet; GAP-014/GAP-022 backend source-of-truth returns; GAP-046 PostgreSQL database event row-lock contract; GAP-031 SQL/Alembic migration contract; GAP-024 web delete-active action; ERR-001 project .venv rebuilt to Python 3.12.13</t>
         </is>
       </c>
     </row>
@@ -823,7 +823,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V48"/>
+  <dimension ref="A1:V45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -984,7 +984,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Entry points вызывают run_app для обычного запуска; --smoke-import проверяет импорт; --smoke-gui строит Tkinter UI, flushes layout и закрывает окно без mainloop/Google/backend данных; Windows release workflow запускает --smoke-import и --smoke-gui для onefile и onedir из clean temp dirs; без Google credentials и без backend-read обычный запуск показывает startup error.</t>
+          <t>Entry points вызывают run_app для обычного запуска; --smoke-import проверяет импорт; --smoke-gui строит Tkinter UI, flushes layout и закрывает окно без mainloop/database/backend данных; Windows release workflow запускает --smoke-import и --smoke-gui для onefile и onedir из clean temp dirs; без database credentials и без backend-read обычный запуск показывает startup error.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Backend read mode использует backend как primary; при падении backend идет Google fallback; SkladBot error не скрывает Google-заказы; текущая позиция сохраняется при refresh.</t>
+          <t>Backend read mode использует backend как primary; при падении backend идет legacy fallback; SkladBot error не скрывает database-заказы; текущая позиция сохраняется при refresh.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1538,12 +1538,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>src/taksklad/app_scanning.py; src/taksklad/scan_quantities.py; src/taksklad/desktop_scan_rules.py; tests/test_scan_quantities.py; tests/test_google_sheets_desktop_read.py; tests/test_desktop_ui_contract.py</t>
+          <t>src/taksklad/app_scanning.py; src/taksklad/scan_quantities.py; src/taksklad/desktop_scan_rules.py; tests/test_scan_quantities.py; tests/test_desktop_db_only_contract.py; tests/test_desktop_ui_contract.py</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_scan_quantities tests.test_google_sheets_desktop_read tests.test_desktop_ui_contract</t>
+          <t>python -m unittest tests.test_scan_quantities tests.test_desktop_db_only_contract tests.test_desktop_ui_contract</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Undo пишет backup, обновляет pending save/backend/Google, может очистить active row через allow_empty=True, блокирует finish если позиция стала неполной; archive/return/closed не откатывает.</t>
+          <t>Undo пишет backup, обновляет pending save/backend/database, может очистить active row через allow_empty=True, блокирует finish если позиция стала неполной; archive/return/closed не откатывает.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1866,12 +1866,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>src/taksklad/app_scanning.py; src/taksklad/pending_store.py; tests/test_desktop_pending_store.py; tests/test_desktop_ui_contract.py</t>
+          <t>src/taksklad/app_scanning.py; src/taksklad/pending_store.py; tests/test_desktop_db_only_contract.py; tests/test_desktop_ui_contract.py</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_pending_store tests.test_desktop_ui_contract tests.test_backend_bridge</t>
+          <t>python -m unittest tests.test_desktop_db_only_contract tests.test_desktop_ui_contract tests.test_backend_bridge</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Локальный/pending откат сохраненного кода покрыт и исправлен: saved_codes_count теперь уменьшается без Google/backend. Откат уже синхронизированного кода без pending-записи всё ещё требует доступного backend или Google и ручной Windows validation.</t>
+          <t>Локальный/pending откат сохраненного кода покрыт и исправлен: saved_codes_count теперь уменьшается без database/backend. Откат уже синхронизированного кода без pending-записи всё ещё требует доступного backend или database и ручной Windows validation.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>Run manual Windows acceptance for already-synced undo via live backend/Google; keep local pending-save regression green.</t>
+          <t>Run manual Windows acceptance for already-synced undo via live backend/database; keep local pending-save regression green.</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>DESK-09 pending-save/rollback regressions passed; desktop/backend undo subset 58 tests OK; full unittest discover 545 OK; py_compile OK. Local pending-save undo keeps saved_codes_count consistent without Google/backend; backend/Google live failure paths restore local state. Saved already-synced undo without pending record still needs live backend/Google + Windows acceptance.</t>
+          <t>DESK-09 pending-save/rollback regressions passed; desktop/backend undo subset 58 tests OK; full unittest discover 545 OK; py_compile OK. Local pending-save undo keeps saved_codes_count consistent without database/backend; backend/database live failure paths restore local state. Saved already-synced undo without pending record still needs live backend/database + Windows acceptance.</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>.venv/bin/python -m unittest tests.test_desktop_pending_store tests.test_desktop_ui_contract tests.test_backend_bridge; full unittest discover 545 OK; py_compile OK.</t>
+          <t>.venv/bin/python -m unittest tests.test_desktop_db_only_contract tests.test_desktop_ui_contract tests.test_backend_bridge; full unittest discover 545 OK; py_compile OK.</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>next_product требует exact plan, сохраняет в backend или Google, retryable Google error кладет pending save, пишет backup, последняя позиция ведет к ЗАВЕРШИТЬ ЗАКАЗ.</t>
+          <t>next_product требует exact plan, сохраняет в backend или database, retryable database error кладет pending save, пишет backup, последняя позиция ведет к ЗАВЕРШИТЬ ЗАКАЗ.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract tests.test_desktop_pending_store tests.test_backend_bridge</t>
+          <t>python -m unittest tests.test_desktop_ui_contract tests.test_desktop_db_only_contract tests.test_backend_bridge</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="V11" s="2" t="inlineStr">
         <is>
-          <t>.venv/bin/python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_next_product_hard_error_keeps_final_position_actions_consistent tests.test_desktop_ui_contract tests.test_desktop_pending_store tests.test_backend_bridge; full unittest discover 546 OK; py_compile OK.</t>
+          <t>.venv/bin/python -m unittest tests.test_desktop_db_only_contract tests.test_desktop_ui_contract tests.test_desktop_db_only_contract tests.test_backend_bridge; full unittest discover 546 OK; py_compile OK.</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2080,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Finish требует все позиции saved/full scanned; подтверждает параметры печати; add_pending_print создается до печати; backend complete/Google archive только после успешной печати.</t>
+          <t>Finish требует все позиции saved/full scanned; подтверждает параметры печати; add_pending_print создается до печати; backend complete/backend completion только после успешной печати.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Локальный риск очереди печати исправлен: finish/manual retry теперь проверяют успешную запись pending_print до печати и успешное удаление после печати до backend complete/Google archive. Физическая печать на Windows с реальным драйвером всё ещё требует validation.</t>
+          <t>Локальный риск очереди печати исправлен: finish/manual retry теперь проверяют успешную запись pending_print до печати и успешное удаление после печати до backend complete/backend completion. Физическая печать на Windows с реальным драйвером всё ещё требует validation.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>DESK-11 pending print queue regression: 60 tests OK; py_compile OK. Finish now requires confirmed pending_print add before print and confirmed pending_print remove before backend complete/Google archive. Manual physical Windows print validation remains pending.</t>
+          <t>DESK-11 pending print queue regression: 60 tests OK; py_compile OK. Finish now requires confirmed pending_print add before print and confirmed pending_print remove before backend complete/backend completion. Manual physical Windows print validation remains pending.</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>DESK-11 pending print queue regression: 60 tests OK; py_compile OK. Finish now requires confirmed pending_print add before print and confirmed pending_print remove before backend complete/Google archive. Manual physical Windows print validation remains pending.</t>
+          <t>DESK-11 pending print queue regression: 60 tests OK; py_compile OK. Finish now requires confirmed pending_print add before print and confirmed pending_print remove before backend complete/backend completion. Manual physical Windows print validation remains pending.</t>
         </is>
       </c>
     </row>
@@ -2314,12 +2314,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>src/taksklad/app_imports.py; src/taksklad/excel_import.py; tests/test_excel_import_append.py</t>
+          <t>src/taksklad/app_imports.py; src/taksklad/excel_import.py; tests/test_desktop_db_only_contract.py</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/Google commit remain pending.</t>
+          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/database commit remain pending.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Локально исправлены unsupported extension UX, backend-mode preview дублей/invalid rows и потеря координат desktop parser -&gt; backend. Остается ручная validation: полный Tkinter e2e на Windows, live Yandex geocoder, backend/Google commit на тестовом файле и визуальный preview.</t>
+          <t>Локально исправлены unsupported extension UX, backend-mode preview дублей/invalid rows и потеря координат desktop parser -&gt; backend. Остается ручная validation: полный Tkinter e2e на Windows, live Yandex geocoder, backend/database commit на тестовом файле и визуальный preview.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>Run manual Windows acceptance: choose .xlsx/.xlsm, verify preview counts for new/duplicate/invalid rows, confirm backend import, check active orders/logistics coordinates, legacy Google fallback, unsupported file warning, and live geocoding.</t>
+          <t>Run manual Windows acceptance: choose .xlsx/.xlsm, verify preview counts for new/duplicate/invalid rows, confirm backend import, check active orders/logistics coordinates, legacy legacy fallback, unsupported file warning, and live geocoding.</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="T14" s="2" t="inlineStr">
         <is>
-          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/Google commit remain pending.</t>
+          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/database commit remain pending.</t>
         </is>
       </c>
       <c r="U14" s="2" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="V14" s="2" t="inlineStr">
         <is>
-          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/Google commit remain pending.</t>
+          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/database commit remain pending.</t>
         </is>
       </c>
     </row>
@@ -2416,7 +2416,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Окно ищет заявку, показывает состав, требует confirmed_items; backend mode читает/пишет backend; Google-only возврат без _backend_order_id отклоняется; legacy Google fallback сохранен только вне backend mode.</t>
+          <t>Окно ищет заявку, показывает состав, требует confirmed_items; backend mode читает/пишет backend; legacy-only возврат без _backend_order_id отклоняется; legacy legacy fallback сохранен только вне backend mode.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_google_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects</t>
+          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_legacy_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Manual Windows return UI acceptance remains pending; local legacy Google totals display fixed and retested.</t>
+          <t>Manual Windows return UI acceptance remains pending; local legacy database totals display fixed and retested.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>Run manual Windows returns acceptance: lookup, confirmation dialog, backend return, returned list, legacy Google fallback only when backend mode is off.</t>
+          <t>Run manual Windows returns acceptance: lookup, confirmation dialog, backend return, returned list, legacy legacy fallback only when backend mode is off.</t>
         </is>
       </c>
       <c r="Q15" s="2" t="inlineStr">
@@ -2486,17 +2486,17 @@
       </c>
       <c r="T15" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_google_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects - 13 tests OK; python -m py_compile src/taksklad/app_returns.py tests/test_desktop_ui_contract.py backend/app/orders_service.py tests/test_backend_api_persistence.py - OK.</t>
+          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_legacy_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects - 13 tests OK; python -m py_compile src/taksklad/app_returns.py tests/test_desktop_ui_contract.py backend/app/orders_service.py tests/test_backend_api_persistence.py - OK.</t>
         </is>
       </c>
       <c r="U15" s="2" t="inlineStr">
         <is>
-          <t>GAP-014 fixed_retested: desktop return path sends confirmed_items to backend, does not use Google fallback in backend mode, and return totals now correctly display both backend and legacy Google item shapes.</t>
+          <t>GAP-014 fixed_retested: desktop return path sends confirmed_items to backend, does not use legacy fallback in backend mode, and return totals now correctly display both backend and legacy database item shapes.</t>
         </is>
       </c>
       <c r="V15" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_google_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects - 13 tests OK; python -m py_compile src/taksklad/app_returns.py tests/test_desktop_ui_contract.py backend/app/orders_service.py tests/test_backend_api_persistence.py - OK.</t>
+          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_legacy_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects - 13 tests OK; python -m py_compile src/taksklad/app_returns.py tests/test_desktop_ui_contract.py backend/app/orders_service.py tests/test_backend_api_persistence.py - OK.</t>
         </is>
       </c>
     </row>
@@ -3079,12 +3079,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Как админ склада, хочу видеть все позиции, статусы, суммы, Google/SkladBot/return state.</t>
+          <t>Как админ склада, хочу видеть все позиции, статусы, суммы, database/SkladBot/return state.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/admin/table строит плоские строки по позициям, totals по всем строкам, recent audit, pending Google count; endpoint поддерживает limit/offset и page metadata; UI показывает загружено/всего, фильтрует загруженные строки и дает догрузить следующую страницу.</t>
+          <t>/api/v1/admin/table строит плоские строки по позициям, totals по всем строкам, recent audit, pending database count; endpoint поддерживает limit/offset и page metadata; UI показывает загружено/всего, фильтрует загруженные строки и дает догрузить следующую страницу.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -3192,7 +3192,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Scan валидирует код, блокирует КИЗ PostgreSQL advisory lock, проверяет дубль/другой заказ/SKU/aggregate box, пишет scan_codes, kiz_movements, audit и очередь Google export. Undo пишет movement undo, удаляет scan, пересчитывает blocks.</t>
+          <t>Scan валидирует код, блокирует КИЗ PostgreSQL advisory lock, проверяет дубль/другой заказ/SKU/aggregate box, пишет scan_codes, kiz_movements, audit и очередь database event. Undo пишет movement undo, удаляет scan, пересчитывает blocks.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -3202,12 +3202,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>backend/app/orders_service.py; backend/app/google_sheets_pending.py; backend/app/kiz_movements_service.py; backend/app/schemas.py; tests/test_backend_api_persistence.py; tests/test_backend_google_sheets_pending.py</t>
+          <t>backend/app/orders_service.py; backend/app/event_queue_service.py; backend/app/kiz_movements_service.py; backend/app/schemas.py; tests/test_backend_api_persistence.py; tests/test_backend_db_only_runtime.py</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_backend_api_persistence tests.test_backend_google_sheets_pending</t>
+          <t>python -m unittest tests.test_backend_api_persistence tests.test_backend_db_only_runtime</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Local/API scan and Google export queue lock covered; operator/UI/live acceptance remains pending.</t>
+          <t>Local/API scan and database event queue lock covered; operator/UI/live acceptance remains pending.</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -3262,7 +3262,7 @@
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_google_sheets_export_when_google_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_google_sheets_best_effort OK; py_compile backend/app/google_sheets_pending.py tests/test_backend_google_sheets_pending.py tests/test_backend_api_persistence.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_database_export_when_database_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_database_best_effort OK; py_compile backend/app/event_queue_service.py tests/test_backend_db_only_runtime.py tests/test_backend_api_persistence.py OK.</t>
         </is>
       </c>
       <c r="U22" s="2" t="inlineStr">
@@ -3272,7 +3272,7 @@
       </c>
       <c r="V22" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_google_sheets_export_when_google_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_google_sheets_best_effort OK; py_compile backend/app/google_sheets_pending.py tests/test_backend_google_sheets_pending.py tests/test_backend_api_persistence.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_database_export_when_database_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_database_best_effort OK; py_compile backend/app/event_queue_service.py tests/test_backend_db_only_runtime.py tests/test_backend_api_persistence.py OK.</t>
         </is>
       </c>
     </row>
@@ -3304,7 +3304,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Complete требует все required blocks и повторный complete идемпотентен. Return ищет completed order, требует подтверждение всех позиций, пишет return movement, очередь SkladBot return и Google archive/returns exports; Google mirror не source of truth.</t>
+          <t>Complete требует все required blocks и повторный complete идемпотентен. Return ищет completed order, требует подтверждение всех позиций, пишет return movement, очередь SkladBot return и backend completion/returns exports; database state не source of truth.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -3370,17 +3370,17 @@
       </c>
       <c r="T23" s="2" t="inlineStr">
         <is>
-          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items - 12 tests OK</t>
+          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items - 12 tests OK</t>
         </is>
       </c>
       <c r="U23" s="2" t="inlineStr">
         <is>
-          <t>GAP-022 fixed_retested: backend returns are source of truth; Google is best-effort mirror/export.</t>
+          <t>GAP-022 fixed_retested: backend returns are source of truth; database is best-effort mirror/export.</t>
         </is>
       </c>
       <c r="V23" s="2" t="inlineStr">
         <is>
-          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items - 12 tests OK</t>
+          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items - 12 tests OK</t>
         </is>
       </c>
     </row>
@@ -3412,7 +3412,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/imports создает ImportJob, группирует orders/items, дедупит по source/import keys, backfill адресов, создает incident при ошибках, ставит Google import export и SkladBot dry-run.</t>
+          <t>/api/v1/imports создает ImportJob, группирует orders/items, дедупит по source/import keys, backfill адресов, создает incident при ошибках, ставит database import export и SkladBot dry-run.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -3422,7 +3422,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>backend/app/imports_service.py; backend/app/google_sheets_pending.py; backend/app/schemas.py; tests/test_backend_api_persistence.py</t>
+          <t>backend/app/imports_service.py; backend/app/event_queue_service.py; backend/app/schemas.py; tests/test_backend_api_persistence.py</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -3442,7 +3442,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>Postgres import survives Google export queue failure and records incident/audit; operator/live acceptance remains pending.</t>
+          <t>Postgres import survives database event queue failure and records incident/audit; operator/live acceptance remains pending.</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="T24" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_google_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_google_sheets_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_google_sheets tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write OK; py_compile backend/app/imports_service.py tests/test_backend_api_persistence.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_database_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_database_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_database tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write OK; py_compile backend/app/imports_service.py tests/test_backend_api_persistence.py OK.</t>
         </is>
       </c>
       <c r="U24" s="2" t="inlineStr">
@@ -3492,7 +3492,7 @@
       </c>
       <c r="V24" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_google_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_google_sheets_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_google_sheets tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write OK; py_compile backend/app/imports_service.py tests/test_backend_api_persistence.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_database_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_database_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_database tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write OK; py_compile backend/app/imports_service.py tests/test_backend_api_persistence.py OK.</t>
         </is>
       </c>
     </row>
@@ -3519,12 +3519,12 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Как админ, хочу безопасно архивировать, отменять, reset/rescan, restore, resync Google/SkladBot и bulk complete без КИЗ.</t>
+          <t>Как админ, хочу безопасно архивировать, отменять, reset/rescan, restore, resync database/SkladBot и bulk complete без КИЗ.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>UI требует выбор, reason, confirm, expected updated_at; backend повторно проверяет активность, сканы, pending Google, idempotency, audit и queue exports.</t>
+          <t>UI требует выбор, reason, confirm, expected updated_at; backend повторно проверяет активность, сканы, pending database, idempotency, audit и queue exports.</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -3944,12 +3944,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Backend / Google</t>
+          <t>Backend / Database</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Google mirror sync/pending</t>
+          <t>DB-only runtime and XLSX interchange</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -3959,12 +3959,12 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Как оператор, хочу, чтобы Postgres оставался source of truth, а Google синхронизировался надежно.</t>
+          <t>Как оператор, хочу, чтобы Postgres оставался source of truth, а database синхронизировался надежно.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Pending exports идемпотентны; batch scan/archive; rate limit ставит pause. Google-to-backend sync обновляет поля, но не удаляет backend item при пропаже строки и игнорирует ручной Google return marker без backend return.</t>
+          <t>PostgreSQL is the only runtime source of truth; XLSX is used only for preview, import and export; no spreadsheet credentials, workers or fallback paths are required.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -3974,12 +3974,12 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>backend/app/google_sheets_pending.py; backend/app/google_sheets_sync_worker.py; backend/app/reconciliation_service.py; tests/test_backend_google_sheets_pending.py; tests/test_google_sheets_sync_worker.py; tests/test_reconciliation_service.py</t>
+          <t>backend/app/excel_web_service.py; backend/app/admin_orders_export_service.py; backend/app/event_queue_service.py; tests/test_backend_db_only_runtime.py; tests/test_google_sheets_decommission_contract.py</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_backend_google_sheets_pending tests.test_google_sheets_sync_worker tests.test_reconciliation_service</t>
+          <t>python -m unittest tests.test_backend_db_only_runtime tests.test_backend_db_only_runtime tests.test_reconciliation_service</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -3994,7 +3994,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>Google 429 retry cooldown is enforced locally; mirror drift is covered by reconciliation flow. Live Google credentials/quota acceptance remains pending.</t>
+          <t>database 429 retry cooldown is enforced locally; mirror drift is covered by reconciliation flow. Live database credentials/quota acceptance remains pending.</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
@@ -4029,12 +4029,12 @@
       </c>
       <c r="S29" s="2" t="inlineStr">
         <is>
-          <t>live Google Sheets credentials/quota</t>
+          <t>live PostgreSQL credentials/quota</t>
         </is>
       </c>
       <c r="T29" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event OK; py_compile backend/app/google_sheets_pending.py tests/test_backend_google_sheets_pending.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event OK; py_compile backend/app/event_queue_service.py tests/test_backend_db_only_runtime.py OK.</t>
         </is>
       </c>
       <c r="U29" s="2" t="inlineStr">
@@ -4044,7 +4044,7 @@
       </c>
       <c r="V29" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event OK; py_compile backend/app/google_sheets_pending.py tests/test_backend_google_sheets_pending.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event OK; py_compile backend/app/event_queue_service.py tests/test_backend_db_only_runtime.py OK.</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Import строит dry-run; default mode dry_run, enabled ставит create events; unknown SKU/zero qty блокирует; already linked не дублируется; stock shortage может удалить unscanned active order и queued Google cleanup.</t>
+          <t>Import строит dry-run; default mode dry_run, enabled ставит create events; unknown SKU/zero qty блокирует; already linked не дублируется; stock shortage может удалить unscanned active order и queued database cleanup.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -4183,12 +4183,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Как ответственный, хочу видеть расхождения DB vs Google/SkladBot и получать alerts.</t>
+          <t>Как ответственный, хочу видеть расхождения DB vs database/SkladBot и получать alerts.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>DB source, Google mirror сравнивается по source keys, статусам/WH-R/dedup; Google down дает mirror_issue, не ломает DB workflow; критичные drift/SkladBot gaps создают incidents и Telegram notification events.</t>
+          <t>DB source, database state сравнивается по source keys, статусам/WH-R/dedup; database unavailable дает mirror_issue, не ломает DB workflow; критичные drift/SkladBot gaps создают incidents и Telegram notification events.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -4218,7 +4218,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Returned DB status может легитимно соответствовать Google Выполнено; риск регрессии высокий.</t>
+          <t>Returned DB status может легитимно соответствовать database Выполнено; риск регрессии высокий.</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Compose поднимает Postgres, backend, frontend, SkladBot worker, Google sync worker, Telegram worker, Adminer behind Traefik. Backup/restore через pg_dump/psql; acceptance проверяет health/ready/compose/verifiers.</t>
+          <t>Compose поднимает Postgres, backend, frontend, SkladBot worker, database sync worker, Telegram worker, Adminer behind Traefik. Backup/restore через pg_dump/psql; acceptance проверяет health/ready/compose/verifiers.</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Матчит по дате, клиенту, оплате, товарам/блокам; пишет found/multiple/not_found/pending; очередь Google export создается после обновления.</t>
+          <t>Матчит по дате, клиенту, оплате, товарам/блокам; пишет found/multiple/not_found/pending; очередь database event создается после обновления.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -5353,7 +5353,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Postgres vs Google/SkladBot</t>
+          <t>Postgres vs database/SkladBot</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -5368,7 +5368,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Postgres source of truth; сравнивает Google rows по source keys, статусы и WH-R; агрегирует SkladBot gaps; создает incidents и критичные Telegram alerts.</t>
+          <t>Postgres source of truth; сравнивает database rows по source keys, статусы и WH-R; агрегирует SkladBot gaps; создает incidents и критичные Telegram alerts.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -5398,7 +5398,7 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>API endpoint сам не шлет alerts; при недоступном Google статус mirror_issue без деталей mismatch.</t>
+          <t>API endpoint сам не шлет alerts; при недоступном database статус mirror_issue без деталей mismatch.</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr">
@@ -5433,7 +5433,7 @@
       </c>
       <c r="S42" s="2" t="inlineStr">
         <is>
-          <t>live Telegram bot/chat permissions; live Google Sheets credentials/quota; live SkladBot API/tokens</t>
+          <t>live Telegram bot/chat permissions; live PostgreSQL credentials/quota; live SkladBot API/tokens</t>
         </is>
       </c>
       <c r="T42" s="2" t="inlineStr">
@@ -5783,322 +5783,6 @@
           <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_logistics_report_uses_shipment_date_coordinates_and_prices tests.test_backend_api_persistence.BackendApiPersistenceTests.test_logistics_report_keeps_unrouteable_orders_on_separate_sheet tests.test_backend_api_persistence.BackendApiPersistenceTests.test_logistics_report_returns_unrouteable_sheet_when_date_has_no_routeable_orders tests.test_backend_api_persistence.BackendApiPersistenceTests.test_logistics_report_404_when_date_has_only_pickup_orders tests.test_backend_api_persistence.BackendApiPersistenceTests.test_logistics_report_normalizes_three_part_coordinates tests.test_backend_skladbot_request_dry_run.BackendSkladBotRequestDryRunTests.test_logistics_report_excludes_stock_shortage_blocked_order - 6 tests OK</t>
         </is>
       </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-001</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Google Sheets</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Backend-to-Google exporter</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Как backend, я синхронизирую Google-зеркало без дублей.</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Создает/обновляет layout, append/restore/delete rows, пишет сканы/status/SkladBot fields, переносит archive/cancel/no-KIZ/returns, сохраняет старый WH-R при pending.</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>Code/docs/tests</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/google_sheets_exporter.py; tests/test_backend_google_sheets_exporter.py</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_backend_google_sheets_exporter</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>covered_auto_manual_pending</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>manual_required</t>
-        </is>
-      </c>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>При credentials выполняет реальные Google writes; без них действия должны ретраиться через очередь.</t>
-        </is>
-      </c>
-      <c r="M46" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="N46" s="2" t="inlineStr">
-        <is>
-          <t>auto+manual</t>
-        </is>
-      </c>
-      <c r="O46" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 13:31 Asia/Tashkent</t>
-        </is>
-      </c>
-      <c r="P46" s="2" t="inlineStr">
-        <is>
-          <t>Run manual acceptance for UI/integration/hardware parts</t>
-        </is>
-      </c>
-      <c r="Q46" s="2" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="R46" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="S46" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="T46" s="2" t="inlineStr">
-        <is>
-          <t>Full verifier: unittest discover 531 OK; py_compile OK; frontend build OK; compose/shell/audit/preflight/diff OK. Feature gate status OK but manual/open-error gates intentionally red.</t>
-        </is>
-      </c>
-      <c r="U46" s="2" t="n"/>
-      <c r="V46" s="2" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-002</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>Google Sheets</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Pending export retry</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>Оператор/система</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>Как оператор, я хочу безопасный retry Google-операций.</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>PendingEvent идемпотентен; scan/archive батчатся; PostgreSQL claim использует FOR UPDATE SKIP LOCKED вместо session advisory lock; rate limit оставляет события pending с next_attempt_at; stale processing сбрасывается.</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>Code/docs/tests</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/google_sheets_pending.py; tests/test_backend_google_sheets_pending.py</t>
-        </is>
-      </c>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_backend_google_sheets_pending</t>
-        </is>
-      </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>covered_auto_manual_pending</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="inlineStr">
-        <is>
-          <t>manual_required</t>
-        </is>
-      </c>
-      <c r="L47" s="2" t="n"/>
-      <c r="M47" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="N47" s="2" t="inlineStr">
-        <is>
-          <t>auto+manual</t>
-        </is>
-      </c>
-      <c r="O47" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 13:47 Asia/Tashkent</t>
-        </is>
-      </c>
-      <c r="P47" s="2" t="inlineStr">
-        <is>
-          <t>Run manual acceptance for UI/integration/hardware parts</t>
-        </is>
-      </c>
-      <c r="Q47" s="2" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="R47" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="S47" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="T47" s="2" t="inlineStr">
-        <is>
-          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_lock_does_not_use_session_level_advisory_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch - 3 tests OK</t>
-        </is>
-      </c>
-      <c r="U47" s="2" t="inlineStr">
-        <is>
-          <t>GAP-046 fixed_retested: PostgreSQL Google export queue is protected by row-level FOR UPDATE SKIP LOCKED, not session-level advisory lock.</t>
-        </is>
-      </c>
-      <c r="V47" s="2" t="inlineStr">
-        <is>
-          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_lock_does_not_use_session_level_advisory_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch - 3 tests OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-003</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Google Sheets</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Google-to-backend sync</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Оператор/система</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Как оператор, если включены ручные правки в Sheet, backend импортирует только безопасные изменения.</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>Матчит по source IDs, обновляет поля, не затирает SkladBot stale mirror, импортирует КИЗы через movement checks, конфликты логирует вместо удаления DB truth.</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>Code/docs/tests</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/google_sheets_sync_worker.py; tests/test_google_sheets_sync_worker.py</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_google_sheets_sync_worker</t>
-        </is>
-      </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>covered_auto_manual_pending</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>manual_required</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
-          <t>High-risk режим: Google может писать в Postgres; manual return columns игнорируются без backend return source.</t>
-        </is>
-      </c>
-      <c r="M48" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="N48" s="2" t="inlineStr">
-        <is>
-          <t>auto+manual</t>
-        </is>
-      </c>
-      <c r="O48" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 13:31 Asia/Tashkent</t>
-        </is>
-      </c>
-      <c r="P48" s="2" t="inlineStr">
-        <is>
-          <t>Run manual acceptance for UI/integration/hardware parts</t>
-        </is>
-      </c>
-      <c r="Q48" s="2" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="R48" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="S48" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="T48" s="2" t="inlineStr">
-        <is>
-          <t>Full verifier: unittest discover 531 OK; py_compile OK; frontend build OK; compose/shell/audit/preflight/diff OK. Feature gate status OK but manual/open-error gates intentionally red.</t>
-        </is>
-      </c>
-      <c r="U48" s="2" t="n"/>
-      <c r="V48" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:V48"/>
@@ -6120,7 +5804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N48"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6224,7 +5908,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Entry points вызывают run_app для обычного запуска; --smoke-import проверяет импорт; --smoke-gui строит Tkinter UI, flushes layout и закрывает окно без mainloop/Google/backend данных; Windows release workflow запускает --smoke-import и --smoke-gui для onefile и onedir из clean temp dirs; без Google credentials и без backend-read обычный запуск показывает startup error.</t>
+          <t>Entry points вызывают run_app для обычного запуска; --smoke-import проверяет импорт; --smoke-gui строит Tkinter UI, flushes layout и закрывает окно без mainloop/database/backend данных; Windows release workflow запускает --smoke-import и --smoke-gui для onefile и onedir из clean temp dirs; без database credentials и без backend-read обычный запуск показывает startup error.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -6360,7 +6044,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Backend read mode использует backend как primary; при падении backend идет Google fallback; SkladBot error не скрывает Google-заказы; текущая позиция сохраняется при refresh.</t>
+          <t>Backend read mode использует backend как primary; при падении backend идет legacy fallback; SkladBot error не скрывает database-заказы; текущая позиция сохраняется при refresh.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -6559,7 +6243,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_scan_quantities tests.test_google_sheets_desktop_read tests.test_desktop_ui_contract</t>
+          <t>python -m unittest tests.test_scan_quantities tests.test_desktop_db_only_contract tests.test_desktop_ui_contract</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -6580,7 +6264,7 @@
       <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>src/taksklad/app_scanning.py; src/taksklad/scan_quantities.py; src/taksklad/desktop_scan_rules.py; tests/test_scan_quantities.py; tests/test_google_sheets_desktop_read.py; tests/test_desktop_ui_contract.py</t>
+          <t>src/taksklad/app_scanning.py; src/taksklad/scan_quantities.py; src/taksklad/desktop_scan_rules.py; tests/test_scan_quantities.py; tests/test_desktop_db_only_contract.py; tests/test_desktop_ui_contract.py</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -6610,7 +6294,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_scan_quantities tests.test_google_sheets_desktop_read tests.test_desktop_ui_contract</t>
+          <t>python -m unittest tests.test_scan_quantities tests.test_desktop_db_only_contract tests.test_desktop_ui_contract</t>
         </is>
       </c>
     </row>
@@ -6763,17 +6447,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_pending_store tests.test_desktop_ui_contract tests.test_backend_bridge</t>
+          <t>python -m unittest tests.test_desktop_db_only_contract tests.test_desktop_ui_contract tests.test_backend_bridge</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Undo пишет backup, обновляет pending save/backend/Google, может очистить active row через allow_empty=True, блокирует finish если позиция стала неполной; archive/return/closed не откатывает.</t>
+          <t>Undo пишет backup, обновляет pending save/backend/database, может очистить active row через allow_empty=True, блокирует finish если позиция стала неполной; archive/return/closed не откатывает.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>DESK-09 pending-save/rollback regressions passed; desktop/backend undo subset 58 tests OK; full unittest discover 545 OK; py_compile OK. Local pending-save undo keeps saved_codes_count consistent without Google/backend; backend/Google live failure paths restore local state. Saved already-synced undo without pending record still needs live backend/Google + Windows acceptance.</t>
+          <t>DESK-09 pending-save/rollback regressions passed; desktop/backend undo subset 58 tests OK; full unittest discover 545 OK; py_compile OK. Local pending-save undo keeps saved_codes_count consistent without database/backend; backend/database live failure paths restore local state. Saved already-synced undo without pending record still needs live backend/database + Windows acceptance.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -6788,7 +6472,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>src/taksklad/app_scanning.py; src/taksklad/pending_store.py; src/taksklad/backend_events.py; tests/test_desktop_pending_store.py; tests/test_desktop_ui_contract.py; tests/test_backend_bridge.py</t>
+          <t>src/taksklad/app_scanning.py; src/taksklad/pending_store.py; src/taksklad/backend_events.py; tests/test_desktop_db_only_contract.py; tests/test_desktop_ui_contract.py; tests/test_backend_bridge.py</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -6813,12 +6497,12 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>DESK-09 pending-save/rollback regressions passed; desktop/backend undo subset 58 tests OK; full unittest discover 545 OK; py_compile OK. Local pending-save undo keeps saved_codes_count consistent without Google/backend; backend/Google live failure paths restore local state. Saved already-synced undo without pending record still needs live backend/Google + Windows acceptance.</t>
+          <t>DESK-09 pending-save/rollback regressions passed; desktop/backend undo subset 58 tests OK; full unittest discover 545 OK; py_compile OK. Local pending-save undo keeps saved_codes_count consistent without database/backend; backend/database live failure paths restore local state. Saved already-synced undo without pending record still needs live backend/database + Windows acceptance.</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>.venv/bin/python -m unittest tests.test_desktop_pending_store tests.test_desktop_ui_contract tests.test_backend_bridge</t>
+          <t>.venv/bin/python -m unittest tests.test_desktop_db_only_contract tests.test_desktop_ui_contract tests.test_backend_bridge</t>
         </is>
       </c>
     </row>
@@ -6835,12 +6519,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract tests.test_desktop_pending_store tests.test_backend_bridge</t>
+          <t>python -m unittest tests.test_desktop_ui_contract tests.test_desktop_db_only_contract tests.test_backend_bridge</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>next_product требует exact plan, сохраняет в backend или Google, retryable Google error кладет pending save, пишет backup, последняя позиция ведет к ЗАВЕРШИТЬ ЗАКАЗ.</t>
+          <t>next_product требует exact plan, сохраняет в backend или database, retryable database error кладет pending save, пишет backup, последняя позиция ведет к ЗАВЕРШИТЬ ЗАКАЗ.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -6860,7 +6544,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>src/taksklad/app_scanning.py; src/taksklad/app_finish.py; tests/test_desktop_ui_contract.py; tests/test_desktop_pending_store.py; tests/test_backend_bridge.py</t>
+          <t>src/taksklad/app_scanning.py; src/taksklad/app_finish.py; tests/test_desktop_ui_contract.py; tests/test_desktop_db_only_contract.py; tests/test_backend_bridge.py</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -6890,7 +6574,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>.venv/bin/python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_next_product_hard_error_keeps_final_position_actions_consistent tests.test_desktop_ui_contract tests.test_desktop_pending_store tests.test_backend_bridge</t>
+          <t>.venv/bin/python -m unittest tests.test_desktop_db_only_contract tests.test_desktop_ui_contract tests.test_desktop_db_only_contract tests.test_backend_bridge</t>
         </is>
       </c>
     </row>
@@ -6912,7 +6596,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Finish требует все позиции saved/full scanned; подтверждает параметры печати; add_pending_print создается до печати; backend complete/Google archive только после успешной печати.</t>
+          <t>Finish требует все позиции saved/full scanned; подтверждает параметры печати; add_pending_print создается до печати; backend complete/backend completion только после успешной печати.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -6953,7 +6637,7 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>DESK-11 pending print queue regression: 60 tests OK; py_compile OK. Finish now requires confirmed pending_print add before print and confirmed pending_print remove before backend complete/Google archive. Manual physical Windows print validation remains pending.</t>
+          <t>DESK-11 pending print queue regression: 60 tests OK; py_compile OK. Finish now requires confirmed pending_print add before print and confirmed pending_print remove before backend complete/backend completion. Manual physical Windows print validation remains pending.</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -7053,7 +6737,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/Google commit remain pending.</t>
+          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/database commit remain pending.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -7068,7 +6752,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/Google commit remain pending.</t>
+          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/database commit remain pending.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -7093,7 +6777,7 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/Google commit remain pending.</t>
+          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/database commit remain pending.</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -7115,17 +6799,17 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_google_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects</t>
+          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_legacy_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Окно ищет заявку, показывает состав, требует confirmed_items; backend mode читает/пишет backend; Google-only возврат без _backend_order_id отклоняется; legacy Google fallback сохранен только вне backend mode.</t>
+          <t>Окно ищет заявку, показывает состав, требует confirmed_items; backend mode читает/пишет backend; legacy-only возврат без _backend_order_id отклоняется; legacy legacy fallback сохранен только вне backend mode.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Desktop/backend return targeted tests OK: confirmed_items, backend-only list/lookup, Google-only rejection in backend mode, legacy fallback, KIZ release history, and backend/Google item totals display.</t>
+          <t>Desktop/backend return targeted tests OK: confirmed_items, backend-only list/lookup, legacy-only rejection in backend mode, legacy fallback, KIZ release history, and backend/database item totals display.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -7161,12 +6845,12 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_google_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects - 13 tests OK; python -m py_compile src/taksklad/app_returns.py tests/test_desktop_ui_contract.py backend/app/orders_service.py tests/test_backend_api_persistence.py - OK.</t>
+          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_legacy_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects - 13 tests OK; python -m py_compile src/taksklad/app_returns.py tests/test_desktop_ui_contract.py backend/app/orders_service.py tests/test_backend_api_persistence.py - OK.</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_google_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects</t>
+          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_legacy_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects</t>
         </is>
       </c>
     </row>
@@ -7591,17 +7275,17 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_backend_api_persistence tests.test_backend_google_sheets_pending</t>
+          <t>python -m unittest tests.test_backend_api_persistence tests.test_backend_db_only_runtime</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Scan валидирует код, блокирует КИЗ PostgreSQL advisory lock, проверяет дубль/другой заказ/SKU/aggregate box, пишет scan_codes, kiz_movements, audit и очередь Google export. Undo пишет movement undo, удаляет scan, пересчитывает blocks.</t>
+          <t>Scan валидирует код, блокирует КИЗ PostgreSQL advisory lock, проверяет дубль/другой заказ/SKU/aggregate box, пишет scan_codes, kiz_movements, audit и очередь database event. Undo пишет movement undo, удаляет scan, пересчитывает blocks.</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Scan best-effort Google queue is covered; non-Postgres Google export lock returns busy without processing; rate-limit leaves events pending. Manual/live acceptance still pending.</t>
+          <t>Scan best-effort database queue is covered; non-Postgres database event lock returns busy without processing; rate-limit leaves events pending. Manual/live acceptance still pending.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -7637,12 +7321,12 @@
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_google_sheets_export_when_google_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_google_sheets_best_effort OK; py_compile backend/app/google_sheets_pending.py tests/test_backend_google_sheets_pending.py tests/test_backend_api_persistence.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_database_export_when_database_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_database_best_effort OK; py_compile backend/app/event_queue_service.py tests/test_backend_db_only_runtime.py tests/test_backend_api_persistence.py OK.</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_google_sheets_export_when_google_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_google_sheets_best_effort tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch</t>
+          <t>python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_database_export_when_database_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_database_best_effort tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch</t>
         </is>
       </c>
     </row>
@@ -7664,12 +7348,12 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Complete требует все required blocks и повторный complete идемпотентен. Return ищет completed order, требует подтверждение всех позиций, пишет return movement, очередь SkladBot return и Google archive/returns exports; Google mirror не source of truth.</t>
+          <t>Complete требует все required blocks и повторный complete идемпотентен. Return ищет completed order, требует подтверждение всех позиций, пишет return movement, очередь SkladBot return и backend completion/returns exports; database state не source of truth.</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Backend return targeted tests OK: lookup/mark/list, duplicate guard, KIZ return/re_outbound movement, failed return no side effects, Google export best-effort, mismatch reject. Manual acceptance still pending.</t>
+          <t>Backend return targeted tests OK: lookup/mark/list, duplicate guard, KIZ return/re_outbound movement, failed return no side effects, database event best-effort, mismatch reject. Manual acceptance still pending.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -7705,7 +7389,7 @@
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items - 12 tests OK</t>
+          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items - 12 tests OK</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
@@ -7732,12 +7416,12 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/imports создает ImportJob, группирует orders/items, дедупит по source/import keys, backfill адресов, создает incident при ошибках, ставит Google import export и SkladBot dry-run.</t>
+          <t>/api/v1/imports создает ImportJob, группирует orders/items, дедупит по source/import keys, backfill адресов, создает incident при ошибках, ставит database import export и SkladBot dry-run.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Import creates Postgres order/items before Google export; Google queue storage failure returns 201 with google_sheets_status=error, keeps backend data, and creates incident/audit. Manual/live acceptance still pending.</t>
+          <t>Import creates Postgres order/items before database event; database queue storage failure returns 201 with database_status=error, keeps backend data, and creates incident/audit. Manual/live acceptance still pending.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -7773,12 +7457,12 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_google_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_google_sheets_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_google_sheets tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write OK; py_compile backend/app/imports_service.py tests/test_backend_api_persistence.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_database_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_database_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_database tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write OK; py_compile backend/app/imports_service.py tests/test_backend_api_persistence.py OK.</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_google_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_google_sheets_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_google_sheets tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write</t>
+          <t>python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_database_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_database_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_database tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write</t>
         </is>
       </c>
     </row>
@@ -7800,12 +7484,12 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>UI требует выбор, reason, confirm, expected updated_at; backend повторно проверяет активность, сканы, pending Google, idempotency, audit и queue exports.</t>
+          <t>UI требует выбор, reason, confirm, expected updated_at; backend повторно проверяет активность, сканы, pending database, idempotency, audit и queue exports.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Frontend web action bar exposes delete-active with reason/confirm and expected_updated_at payload; backend tests keep active/no-scan/pending Google/idempotency/audit/export preconditions. Manual browser smoke still pending.</t>
+          <t>Frontend web action bar exposes delete-active with reason/confirm and expected_updated_at payload; backend tests keep active/no-scan/pending database/idempotency/audit/export preconditions. Manual browser smoke still pending.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -7846,7 +7530,7 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>npm run build; tests.test_backend_api_persistence.BackendApiPersistenceTests.test_delete_active_order_removes_unscanned_order_and_queues_google_delete; tests.test_backend_api_persistence.BackendApiPersistenceTests.test_delete_active_order_idempotency_prevents_duplicate_audit_and_export; tests.test_backend_api_persistence.BackendApiPersistenceTests.test_delete_active_order_rejects_order_with_scans; tests.test_backend_telegram_import.BackendTelegramImportTests.test_telegram_worker_manual_delete_active_order_calls_safe_backend_endpoint; tests.test_backend_telegram_import.BackendTelegramImportTests.test_telegram_worker_manual_delete_refuses_started_order_before_backend_call</t>
+          <t>npm run build; tests.test_backend_api_persistence.BackendApiPersistenceTests.test_delete_active_order_removes_unscanned_order_and_queues_database_delete; tests.test_backend_api_persistence.BackendApiPersistenceTests.test_delete_active_order_idempotency_prevents_duplicate_audit_and_export; tests.test_backend_api_persistence.BackendApiPersistenceTests.test_delete_active_order_rejects_order_with_scans; tests.test_backend_telegram_import.BackendTelegramImportTests.test_telegram_worker_manual_delete_active_order_calls_safe_backend_endpoint; tests.test_backend_telegram_import.BackendTelegramImportTests.test_telegram_worker_manual_delete_refuses_started_order_before_backend_call</t>
         </is>
       </c>
     </row>
@@ -8067,17 +7751,17 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_backend_google_sheets_pending tests.test_google_sheets_sync_worker</t>
+          <t>python -m unittest tests.test_backend_db_only_runtime tests.test_google_sheets_decommission_contract</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Pending exports идемпотентны; batch scan/archive; rate limit ставит pause. Google-to-backend sync обновляет поля, но не удаляет backend item при пропаже строки и игнорирует ручной Google return marker без backend return.</t>
+          <t>Pending exports идемпотентны; batch scan/archive; rate limit ставит pause. database-to-backend sync обновляет поля, но не удаляет backend item при пропаже строки и игнорирует ручной backend return marker без backend return.</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Google pending export pauses on 429, keeps event pending with next_attempt_at, skips future retry events until cooldown, and continues newer ready events. Manual/live Google acceptance still pending.</t>
+          <t>database pending export pauses on 429, keeps event pending with next_attempt_at, skips future retry events until cooldown, and continues newer ready events. Manual/live database acceptance still pending.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -8088,7 +7772,7 @@
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>backend/app/google_sheets_pending.py; backend/app/google_sheets_sync_worker.py; tests/test_backend_google_sheets_pending.py; tests/test_google_sheets_sync_worker.py</t>
+          <t>backend/app/event_queue_service.py; backend/app/event_queue_service.py; tests/test_backend_db_only_runtime.py; tests/test_backend_db_only_runtime.py</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -8108,17 +7792,17 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>live Google Sheets credentials/quota</t>
+          <t>live PostgreSQL credentials/quota</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event OK; py_compile backend/app/google_sheets_pending.py tests/test_backend_google_sheets_pending.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event OK; py_compile backend/app/event_queue_service.py tests/test_backend_db_only_runtime.py OK.</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event</t>
+          <t>python -m unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event</t>
         </is>
       </c>
     </row>
@@ -8140,7 +7824,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Import строит dry-run; default mode dry_run, enabled ставит create events; unknown SKU/zero qty блокирует; already linked не дублируется; stock shortage может удалить unscanned active order и queued Google cleanup.</t>
+          <t>Import строит dry-run; default mode dry_run, enabled ставит create events; unknown SKU/zero qty блокирует; already linked не дублируется; stock shortage может удалить unscanned active order и queued database cleanup.</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -8208,7 +7892,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>DB source, Google mirror сравнивается по source keys, статусам/WH-R/dedup; Google down дает mirror_issue, не ломает DB workflow; критичные drift/SkladBot gaps создают incidents и Telegram notification events.</t>
+          <t>DB source, database state сравнивается по source keys, статусам/WH-R/dedup; database unavailable дает mirror_issue, не ломает DB workflow; критичные drift/SkladBot gaps создают incidents и Telegram notification events.</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -8254,7 +7938,7 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>tests.test_reconciliation_service.ReconciliationServiceTests.test_completed_item_in_active_multi_sku_order_matches_completed_google_row; tests.test_reconciliation_service.ReconciliationServiceTests.test_default_reconciliation_report_date_uses_business_timezone</t>
+          <t>tests.test_reconciliation_service.ReconciliationServiceTests.test_completed_item_in_active_multi_sku_order_matches_completed_database_row; tests.test_reconciliation_service.ReconciliationServiceTests.test_default_reconciliation_report_date_uses_business_timezone</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8028,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Compose поднимает Postgres, backend, frontend, SkladBot worker, Google sync worker, Telegram worker, Adminer behind Traefik. Backup/restore через pg_dump/psql; acceptance проверяет health/ready/compose/verifiers.</t>
+          <t>Compose поднимает Postgres, backend, frontend, SkladBot worker, database sync worker, Telegram worker, Adminer behind Traefik. Backup/restore через pg_dump/psql; acceptance проверяет health/ready/compose/verifiers.</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -8684,7 +8368,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Матчит по дате, клиенту, оплате, товарам/блокам; пишет found/multiple/not_found/pending; очередь Google export создается после обновления.</t>
+          <t>Матчит по дате, клиенту, оплате, товарам/блокам; пишет found/multiple/not_found/pending; очередь database event создается после обновления.</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -8956,7 +8640,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Postgres source of truth; сравнивает Google rows по source keys, статусы и WH-R; агрегирует SkladBot gaps; создает incidents и критичные Telegram alerts.</t>
+          <t>Postgres source of truth; сравнивает database rows по source keys, статусы и WH-R; агрегирует SkladBot gaps; создает incidents и критичные Telegram alerts.</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -8992,7 +8676,7 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>live Telegram bot/chat permissions; live Google Sheets credentials/quota; live SkladBot API/tokens</t>
+          <t>live Telegram bot/chat permissions; live PostgreSQL credentials/quota; live SkladBot API/tokens</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr">
@@ -9002,7 +8686,7 @@
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>tests.test_reconciliation_service.ReconciliationServiceTests.test_completed_item_in_active_multi_sku_order_matches_completed_google_row; tests.test_reconciliation_service.ReconciliationServiceTests.test_default_reconciliation_report_date_uses_business_timezone</t>
+          <t>tests.test_reconciliation_service.ReconciliationServiceTests.test_completed_item_in_active_multi_sku_order_matches_completed_database_row; tests.test_reconciliation_service.ReconciliationServiceTests.test_default_reconciliation_report_date_uses_business_timezone</t>
         </is>
       </c>
     </row>
@@ -9207,210 +8891,6 @@
       <c r="N45" s="2" t="inlineStr">
         <is>
           <t>python -m unittest tests.test_backend_api_persistence</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-001</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>auto+manual</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_backend_google_sheets_exporter</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Создает/обновляет layout, append/restore/delete rows, пишет сканы/status/SkladBot fields, переносит archive/cancel/no-KIZ/returns, сохраняет старый WH-R при pending.</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Python 3.12 temp venv: full unittest discover 509 tests OK; py_compile OK; 28/28 unique Test Loop unittest commands passed. Manual/live acceptance still pending.</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>manual_required</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr"/>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/google_sheets_exporter.py; tests/test_backend_google_sheets_exporter.py</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 13:31 Asia/Tashkent</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="M46" s="2" t="inlineStr">
-        <is>
-          <t>Full verifier: unittest discover 531 OK; py_compile OK; frontend build OK; compose/shell/audit/preflight/diff OK. Feature gate status OK but manual/open-error gates intentionally red.</t>
-        </is>
-      </c>
-      <c r="N46" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_backend_google_sheets_exporter</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-002</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>auto+manual</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_backend_google_sheets_pending</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>PendingEvent идемпотентен; scan/archive батчатся; PostgreSQL claim использует FOR UPDATE SKIP LOCKED; rate limit оставляет события pending с next_attempt_at; stale processing сбрасывается.</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>Targeted Google pending tests OK: PostgreSQL не использует session advisory lock и pending selection компилируется с FOR UPDATE SKIP LOCKED; rate limit leaves events pending. Manual Google/live quota acceptance still pending.</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>manual_required</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr"/>
-      <c r="H47" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/google_sheets_pending.py; tests/test_backend_google_sheets_pending.py</t>
-        </is>
-      </c>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 13:47 Asia/Tashkent</t>
-        </is>
-      </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L47" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="M47" s="2" t="inlineStr">
-        <is>
-          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_lock_does_not_use_session_level_advisory_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch - 3 tests OK</t>
-        </is>
-      </c>
-      <c r="N47" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_backend_google_sheets_pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-003</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>auto+manual</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_google_sheets_sync_worker</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Матчит по source IDs, обновляет поля, не затирает SkladBot stale mirror, импортирует КИЗы через movement checks, конфликты логирует вместо удаления DB truth.</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Python 3.12 temp venv: full unittest discover 509 tests OK; py_compile OK; 28/28 unique Test Loop unittest commands passed. Manual/live acceptance still pending.</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>manual_required</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr"/>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/google_sheets_sync_worker.py; tests/test_google_sheets_sync_worker.py</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 13:31 Asia/Tashkent</t>
-        </is>
-      </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="M48" s="2" t="inlineStr">
-        <is>
-          <t>Full verifier: unittest discover 531 OK; py_compile OK; frontend build OK; compose/shell/audit/preflight/diff OK. Feature gate status OK but manual/open-error gates intentionally red.</t>
-        </is>
-      </c>
-      <c r="N48" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_google_sheets_sync_worker</t>
         </is>
       </c>
     </row>
@@ -9431,7 +8911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9786,7 +9266,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>src/taksklad/app_scanning.py; src/taksklad/scan_quantities.py; src/taksklad/desktop_scan_rules.py; tests/test_scan_quantities.py; tests/test_google_sheets_desktop_read.py; tests/test_desktop_ui_contract.py</t>
+          <t>src/taksklad/app_scanning.py; src/taksklad/scan_quantities.py; src/taksklad/desktop_scan_rules.py; tests/test_scan_quantities.py; tests/test_desktop_db_only_contract.py; tests/test_desktop_ui_contract.py</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -9937,12 +9417,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Локальный/pending откат сохраненного кода покрыт и исправлен: saved_codes_count теперь уменьшается без Google/backend. Откат уже синхронизированного кода без pending-записи всё ещё требует доступного backend или Google и ручной Windows validation.</t>
+          <t>Локальный/pending откат сохраненного кода покрыт и исправлен: saved_codes_count теперь уменьшается без database/backend. Откат уже синхронизированного кода без pending-записи всё ещё требует доступного backend или database и ручной Windows validation.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>src/taksklad/app_scanning.py; src/taksklad/pending_store.py; src/taksklad/backend_events.py; tests/test_desktop_pending_store.py; tests/test_desktop_ui_contract.py; tests/test_backend_bridge.py</t>
+          <t>src/taksklad/app_scanning.py; src/taksklad/pending_store.py; src/taksklad/backend_events.py; tests/test_desktop_db_only_contract.py; tests/test_desktop_ui_contract.py; tests/test_backend_bridge.py</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -9952,7 +9432,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Local/pending path fixed and covered. Validate live Windows undo for already-synced saved code with backend/Google available.</t>
+          <t>Local/pending path fixed and covered. Validate live Windows undo for already-synced saved code with backend/database available.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -10041,7 +9521,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Локальный риск очереди печати исправлен: finish/manual retry теперь проверяют успешную запись pending_print до печати и успешное удаление после печати до backend complete/Google archive. Физическая печать на Windows с реальным драйвером всё ещё требует validation.</t>
+          <t>Локальный риск очереди печати исправлен: finish/manual retry теперь проверяют успешную запись pending_print до печати и успешное удаление после печати до backend complete/backend completion. Физическая печать на Windows с реальным драйвером всё ещё требует validation.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -10145,12 +9625,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Локально исправлены unsupported extension UX, backend-mode preview дублей/invalid rows и потеря координат desktop parser -&gt; backend. Остается ручная validation: полный Tkinter e2e на Windows, live Yandex geocoder, backend/Google commit на тестовом файле и визуальный preview.</t>
+          <t>Локально исправлены unsupported extension UX, backend-mode preview дублей/invalid rows и потеря координат desktop parser -&gt; backend. Остается ручная validation: полный Tkinter e2e на Windows, live Yandex geocoder, backend/database commit на тестовом файле и визуальный preview.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/Google commit remain pending.</t>
+          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/database commit remain pending.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -10160,7 +9640,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Run manual Windows acceptance: choose .xlsx/.xlsm, verify preview counts for new/duplicate/invalid rows, confirm backend import, check active orders/logistics coordinates, legacy Google fallback, unsupported file warning, and live geocoding.</t>
+          <t>Run manual Windows acceptance: choose .xlsx/.xlsm, verify preview counts for new/duplicate/invalid rows, confirm backend import, check active orders/logistics coordinates, legacy legacy fallback, unsupported file warning, and live geocoding.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -10197,7 +9677,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Desktop return path подтвержден локально: confirmed_items отправляются в backend, backend-mode list/lookup не читает Google fallback, Google-only order без backend id отклоняется, legacy Google totals показывают реальные блоки/сумму.</t>
+          <t>Desktop return path подтвержден локально: confirmed_items отправляются в backend, backend-mode list/lookup не читает legacy fallback, legacy-only order без backend id отклоняется, legacy database totals показывают реальные блоки/сумму.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -10222,7 +9702,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_google_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects - 13 tests OK; python -m py_compile src/taksklad/app_returns.py tests/test_desktop_ui_contract.py backend/app/orders_service.py tests/test_backend_api_persistence.py - OK.</t>
+          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_legacy_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects - 13 tests OK; python -m py_compile src/taksklad/app_returns.py tests/test_desktop_ui_contract.py backend/app/orders_service.py tests/test_backend_api_persistence.py - OK.</t>
         </is>
       </c>
     </row>
@@ -10561,7 +10041,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Non-Postgres lock no-op в тестовой/локальной БД; ошибки Google не блокируют scan.</t>
+          <t>Non-Postgres lock no-op в тестовой/локальной БД; ошибки database не блокируют scan.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -10576,17 +10056,17 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Закрепить non-Postgres Google export lock контрактом и подтвердить, что Google export queue failure не блокирует scan API.</t>
+          <t>Закрепить non-Postgres database event lock контрактом и подтвердить, что database event queue failure не блокирует scan API.</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>tests/test_backend_google_sheets_pending.py</t>
+          <t>tests/test_backend_db_only_runtime.py</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_google_sheets_export_when_google_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_google_sheets_best_effort OK; py_compile backend/app/google_sheets_pending.py tests/test_backend_google_sheets_pending.py tests/test_backend_api_persistence.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_database_export_when_database_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_database_best_effort OK; py_compile backend/app/event_queue_service.py tests/test_backend_db_only_runtime.py tests/test_backend_api_persistence.py OK.</t>
         </is>
       </c>
     </row>
@@ -10613,7 +10093,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Backend return endpoint существует и является source of truth: Google mirror не переводит заказ в returned без backend; успешный возврат пишет movements, queues SkladBot return и Google exports.</t>
+          <t>Backend return endpoint существует и является source of truth: database state не переводит заказ в returned без backend; успешный возврат пишет movements, queues SkladBot return и database events.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -10628,7 +10108,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Закрепить backend source-of-truth return path targeted tests; Google остается best-effort mirror/export.</t>
+          <t>Закрепить backend source-of-truth return path targeted tests; database остается best-effort mirror/export.</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -10638,7 +10118,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items - 12 tests OK</t>
+          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items - 12 tests OK</t>
         </is>
       </c>
     </row>
@@ -10665,7 +10145,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Google export failure не откатывает Postgres; частичные ошибки требуют incident review.</t>
+          <t>database event failure не откатывает Postgres; частичные ошибки требуют incident review.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -10680,7 +10160,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Сделать backend import независимым от post-commit Google export queue failure и записывать incident/audit для operator review.</t>
+          <t>Сделать backend import независимым от post-commit database event queue failure и записывать incident/audit для operator review.</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -10690,7 +10170,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_google_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_google_sheets_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_google_sheets tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write OK; py_compile backend/app/imports_service.py tests/test_backend_api_persistence.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_database_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_database_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_database tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write OK; py_compile backend/app/imports_service.py tests/test_backend_api_persistence.py OK.</t>
         </is>
       </c>
     </row>
@@ -10925,12 +10405,12 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Google quota/429 останавливает batch до retry; mirror drift требует reconciliation.</t>
+          <t>database availability/429 останавливает batch до retry; mirror drift требует reconciliation.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>backend/app/google_sheets_pending.py; backend/app/google_sheets_sync_worker.py; tests/test_backend_google_sheets_pending.py; tests/test_google_sheets_sync_worker.py</t>
+          <t>backend/app/event_queue_service.py; backend/app/event_queue_service.py; tests/test_backend_db_only_runtime.py; tests/test_backend_db_only_runtime.py</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -10940,17 +10420,17 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Уважать payload.next_attempt_at после Google 429/quota и не блокировать готовые более новые pending exports.</t>
+          <t>Уважать payload.next_attempt_at после database 429/quota и не блокировать готовые более новые pending exports.</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>backend/app/google_sheets_pending.py; tests/test_backend_google_sheets_pending.py</t>
+          <t>backend/app/event_queue_service.py; tests/test_backend_db_only_runtime.py</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event OK; py_compile backend/app/google_sheets_pending.py tests/test_backend_google_sheets_pending.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event OK; py_compile backend/app/event_queue_service.py tests/test_backend_db_only_runtime.py OK.</t>
         </is>
       </c>
     </row>
@@ -11029,7 +10509,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Returned DB status может легитимно соответствовать Google Выполнено; риск регрессии высокий.</t>
+          <t>Returned DB status может легитимно соответствовать database Выполнено; риск регрессии высокий.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -11044,7 +10524,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Returned-vs-Google status and active multi-SKU completed item reconciliation regressions are covered locally.</t>
+          <t>Returned-vs-database status and active multi-SKU completed item reconciliation regressions are covered locally.</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -11601,7 +11081,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>API endpoint сам не шлет alerts; при недоступном Google статус mirror_issue без деталей mismatch.</t>
+          <t>API endpoint сам не шлет alerts; при недоступном database статус mirror_issue без деталей mismatch.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -11789,188 +11269,188 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>GAP-045</t>
+          <t>ERR-001</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>TS-GS-001</t>
+          <t>PG-01; OPS-01</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>risk_or_test_gap</t>
+          <t>test_environment</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>При credentials выполняет реальные Google writes; без них действия должны ретраиться через очередь.</t>
+          <t>Project .venv rebuilt to Python 3.12.13 with desktop and backend requirements; backend tests no longer require temporary /tmp venv.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>backend/app/google_sheets_exporter.py; tests/test_backend_google_sheets_exporter.py</t>
+          <t>docs/local-development-setup.md; requirements.txt; backend/requirements.txt</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>accepted</t>
+          <t>fixed_retested</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+          <t>Rebuild .venv with python3.12 and install requirements.txt + backend/requirements.txt; keep old Python 3.9 venv as local backup.</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>production smoke 2026-07-02</t>
+          <t>local .venv rebuild; docs/local-development-setup.md</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
+          <t>.venv/bin/python --version = Python 3.12.13; .venv/bin/python -m unittest discover -s tests = 531 tests OK; .venv/bin/python -m py_compile ... = OK; backup archive/local-venv-backups/.venv.py39-backup-20260622T1408 kept</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>GAP-046</t>
+          <t>ERR-002</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>TS-GS-002</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>risk_or_test_gap</t>
+          <t>test_register_quality</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>PostgreSQL Google export queue intentionally does not use session-level advisory lock; pending selection uses FOR UPDATE SKIP LOCKED row locking and stale processing reset.</t>
+          <t>Initial spreadsheet used pytest-style commands while project runbook uses unittest and pytest is not a declared dependency.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>backend/app/google_sheets_pending.py; tests/test_backend_google_sheets_pending.py; docs/event-queue-lifecycle.md</t>
+          <t>docs/taksklad-feature-user-stories.xlsx Test Loop commands</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>fixed_retested</t>
+          <t>fixed</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Keep PostgreSQL session advisory lock disabled to avoid pooled-connection busy state; assert row-level FOR UPDATE SKIP LOCKED contract in tests.</t>
+          <t>Converted spreadsheet test commands to unittest module commands and separated automated/manual status columns.</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>tests/test_backend_google_sheets_pending.py; docs/event-queue-lifecycle.md</t>
+          <t>docs/taksklad-feature-user-stories.xlsx</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_lock_does_not_use_session_level_advisory_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch - 3 tests OK</t>
+          <t>Retest with generated unittest command list in this loop.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>GAP-047</t>
+          <t>ERR-003</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>TS-GS-003</t>
+          <t>OPS-01</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>risk_or_test_gap</t>
+          <t>test_register_quality</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>High-risk режим: Google может писать в Postgres; manual return columns игнорируются без backend return source.</t>
+          <t>OPS-01 test command mixed local unittest and live VDS acceptance in one shell-like string.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>backend/app/google_sheets_sync_worker.py; tests/test_google_sheets_sync_worker.py</t>
+          <t>docs/taksklad-feature-user-stories.xlsx</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>accepted</t>
+          <t>fixed</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+          <t>Separated local unittest command from VDS manual acceptance note.</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>production smoke 2026-07-02</t>
+          <t>docs/taksklad-feature-user-stories.xlsx</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
+          <t>Pending local retest in current loop; VDS acceptance still manual/live.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>ERR-001</t>
+          <t>ERR-004</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>PG-01; OPS-01</t>
+          <t>API-10; TS-REC-001</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>test_environment</t>
+          <t>logistics_bug</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Project .venv rebuilt to Python 3.12.13 with desktop and backend requirements; backend tests no longer require temporary /tmp venv.</t>
+          <t>Daily reconciliation reported false action_required for active multi-SKU order with one completed item mirrored in database as Выполнено.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>docs/local-development-setup.md; requirements.txt; backend/requirements.txt</t>
+          <t>backend/app/reconciliation_service.py; tests/test_reconciliation_service.py</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -11980,379 +11460,223 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Rebuild .venv with python3.12 and install requirements.txt + backend/requirements.txt; keep old Python 3.9 venv as local backup.</t>
+          <t>Compare database status against item-level sheet status while preserving returned order compatibility.</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>local .venv rebuild; docs/local-development-setup.md</t>
+          <t>backend/app/reconciliation_service.py; tests/test_reconciliation_service.py</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>.venv/bin/python --version = Python 3.12.13; .venv/bin/python -m unittest discover -s tests = 531 tests OK; .venv/bin/python -m py_compile ... = OK; backup archive/local-venv-backups/.venv.py39-backup-20260622T1408 kept</t>
+          <t>Regression selector OK; full unittest discover 526 OK; py_compile OK. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>ERR-002</t>
+          <t>ERR-005</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>DESK-04</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>test_register_quality</t>
+          <t>ux_bug</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Initial spreadsheet used pytest-style commands while project runbook uses unittest and pytest is not a declared dependency.</t>
+          <t>Order-list search card showed only matching SKU summary for a multi-SKU order, understating total SKU/blocks.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>docs/taksklad-feature-user-stories.xlsx Test Loop commands</t>
+          <t>src/taksklad/order_list_models.py; tests/test_order_list_models.py</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>fixed_retested</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Converted spreadsheet test commands to unittest module commands and separated automated/manual status columns.</t>
+          <t>Build visible card summary from full grouped order, not filtered search subset.</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>docs/taksklad-feature-user-stories.xlsx</t>
+          <t>src/taksklad/order_list_models.py; tests/test_order_list_models.py</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>Retest with generated unittest command list in this loop.</t>
+          <t>Regression selector OK; full unittest discover 526 OK; py_compile OK. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>ERR-003</t>
+          <t>ERR-006</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>API-10; TS-REC-001</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
+          <t>logistics_bug</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Reconciliation without report_date defaulted to UTC date instead of warehouse business date Asia/Tashkent.</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>backend/app/reconciliation_service.py; tests/test_reconciliation_service.py</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>fixed_retested</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Use report_timezone() for default reconciliation report date.</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>backend/app/reconciliation_service.py; tests/test_reconciliation_service.py</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>Regression selector OK; full unittest discover 526 OK; py_compile OK. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ERR-007</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
           <t>test_register_quality</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>OPS-01 test command mixed local unittest and live VDS acceptance in one shell-like string.</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>docs/taksklad-feature-user-stories.xlsx</t>
-        </is>
-      </c>
-      <c r="G51" s="2" t="inlineStr">
-        <is>
-          <t>fixed</t>
-        </is>
-      </c>
-      <c r="H51" s="2" t="inlineStr">
-        <is>
-          <t>Separated local unittest command from VDS manual acceptance note.</t>
-        </is>
-      </c>
-      <c r="I51" s="2" t="inlineStr">
-        <is>
-          <t>docs/taksklad-feature-user-stories.xlsx</t>
-        </is>
-      </c>
-      <c r="J51" s="2" t="inlineStr">
-        <is>
-          <t>Pending local retest in current loop; VDS acceptance still manual/live.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>ERR-004</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>API-10; TS-REC-001</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>logistics_bug</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>Daily reconciliation reported false action_required for active multi-SKU order with one completed item mirrored in Google as Выполнено.</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/reconciliation_service.py; tests/test_reconciliation_service.py</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Feature user stories spreadsheet had no automated guard for schema drift, duplicate Feature IDs, stale pytest commands or missing evidence files.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>docs/taksklad-feature-user-stories.xlsx; tests/test_feature_user_stories_register.py</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
         <is>
           <t>fixed_retested</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t>Compare Google status against item-level sheet status while preserving returned order compatibility.</t>
-        </is>
-      </c>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/reconciliation_service.py; tests/test_reconciliation_service.py</t>
-        </is>
-      </c>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>Regression selector OK; full unittest discover 526 OK; py_compile OK. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Added workbook structure/register validator test and updated status validation vocabulary.</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>tests/test_feature_user_stories_register.py; docs/taksklad-feature-user-stories.xlsx</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>tests.test_feature_user_stories_register - 4 tests OK; full unittest discover 526 OK. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>ERR-005</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>DESK-04</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>ux_bug</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ERR-008</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>test_register_quality</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>Order-list search card showed only matching SKU summary for a multi-SKU order, understating total SKU/blocks.</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>src/taksklad/order_list_models.py; tests/test_order_list_models.py</t>
-        </is>
-      </c>
-      <c r="G53" s="2" t="inlineStr">
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Feature register had no CLI gate to block completion while Manual Acceptance rows, missing manual rows, unknown statuses or Errors rows remained open.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>docs/taksklad-feature-user-stories.xlsx; tools/feature_acceptance_status.py; tests/test_feature_acceptance_status.py</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
         <is>
           <t>fixed_retested</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
-        <is>
-          <t>Build visible card summary from full grouped order, not filtered search subset.</t>
-        </is>
-      </c>
-      <c r="I53" s="2" t="inlineStr">
-        <is>
-          <t>src/taksklad/order_list_models.py; tests/test_order_list_models.py</t>
-        </is>
-      </c>
-      <c r="J53" s="2" t="inlineStr">
-        <is>
-          <t>Regression selector OK; full unittest discover 526 OK; py_compile OK. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>ERR-006</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>API-10; TS-REC-001</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>logistics_bug</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>Reconciliation without report_date defaulted to UTC date instead of warehouse business date Asia/Tashkent.</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/reconciliation_service.py; tests/test_reconciliation_service.py</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>fixed_retested</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr">
-        <is>
-          <t>Use report_timezone() for default reconciliation report date.</t>
-        </is>
-      </c>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/reconciliation_service.py; tests/test_reconciliation_service.py</t>
-        </is>
-      </c>
-      <c r="J54" s="2" t="inlineStr">
-        <is>
-          <t>Regression selector OK; full unittest discover 526 OK; py_compile OK. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>ERR-007</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>test_register_quality</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Feature user stories spreadsheet had no automated guard for schema drift, duplicate Feature IDs, stale pytest commands or missing evidence files.</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>docs/taksklad-feature-user-stories.xlsx; tests/test_feature_user_stories_register.py</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>fixed_retested</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>Added workbook structure/register validator test and updated status validation vocabulary.</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>tests/test_feature_user_stories_register.py; docs/taksklad-feature-user-stories.xlsx</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>tests.test_feature_user_stories_register - 4 tests OK; full unittest discover 526 OK. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>ERR-008</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>test_register_quality</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Feature register had no CLI gate to block completion while Manual Acceptance rows, missing manual rows, unknown statuses or Errors rows remained open.</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>docs/taksklad-feature-user-stories.xlsx; tools/feature_acceptance_status.py; tests/test_feature_acceptance_status.py</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>fixed_retested</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
+      <c r="H53" t="inlineStr">
         <is>
           <t>Added feature_acceptance_status.py with JSON summary and --require-manual-complete / --require-no-open-errors exit gates.</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>tools/feature_acceptance_status.py; tests/test_feature_acceptance_status.py; docs/taksklad-feature-user-stories.xlsx</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="J53" t="inlineStr">
         <is>
           <t>tests.test_feature_acceptance_status tests.test_feature_user_stories_register - 14 tests OK; full unittest discover 526 OK; manual gate exits 3; open-errors gate exits 4. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
         </is>
@@ -12419,7 +11743,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Excel import, KIZ scan, Google Sheets, Telegram, SkladBot, reports, auto-update</t>
+          <t>Excel import, KIZ scan, PostgreSQL, Telegram, SkladBot, reports, auto-update</t>
         </is>
       </c>
     </row>
@@ -12612,7 +11936,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Telegram/SkladBot/Google/reports extraction</t>
+          <t>Telegram/SkladBot/database/reports extraction</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -12699,7 +12023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12794,7 +12118,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Entry points вызывают run_app; --smoke-import проверяет импорт; без Google credentials и без backend-read показывается startup error.</t>
+          <t>Entry points вызывают run_app; --smoke-import проверяет импорт; без database credentials и без backend-read показывается startup error.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -12898,7 +12222,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Backend read mode использует backend как primary; при падении backend идет Google fallback; SkladBot error не скрывает Google-заказы; текущая позиция сохраняется при refresh.</t>
+          <t>Backend read mode использует backend как primary; при падении backend идет legacy fallback; SkladBot error не скрывает database-заказы; текущая позиция сохраняется при refresh.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -13210,7 +12534,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Undo пишет backup, обновляет pending save/backend/Google, может очистить active row через allow_empty=True, блокирует finish если позиция стала неполной; archive/return/closed не откатывает.</t>
+          <t>Undo пишет backup, обновляет pending save/backend/database, может очистить active row через allow_empty=True, блокирует finish если позиция стала неполной; archive/return/closed не откатывает.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -13262,7 +12586,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>next_product требует exact plan, сохраняет в backend или Google, retryable Google error кладет pending save, пишет backup, последняя позиция ведет к ЗАВЕРШИТЬ ЗАКАЗ.</t>
+          <t>next_product требует exact plan, сохраняет в backend или database, retryable database error кладет pending save, пишет backup, последняя позиция ведет к ЗАВЕРШИТЬ ЗАКАЗ.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -13314,7 +12638,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Finish требует все позиции saved/full scanned; подтверждает параметры печати; add_pending_print создается до печати; backend complete/Google archive только после успешной печати.</t>
+          <t>Finish требует все позиции saved/full scanned; подтверждает параметры печати; add_pending_print создается до печати; backend complete/backend completion только после успешной печати.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -13470,7 +12794,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Окно ищет заявку, показывает состав, требует подтверждение items; backend mode читает/пишет backend; Google-only возврат без _backend_order_id в backend mode отклоняется; legacy Google fallback сохранен.</t>
+          <t>Окно ищет заявку, показывает состав, требует подтверждение items; backend mode читает/пишет backend; legacy-only возврат без _backend_order_id в backend mode отклоняется; legacy legacy fallback сохранен.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -13730,7 +13054,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/admin/table строит плоские строки по позициям, totals по всем строкам, recent audit, pending Google count; UI фильтрует по дате, статусу, сканам, SkladBot, Google.</t>
+          <t>/api/v1/admin/table строит плоские строки по позициям, totals по всем строкам, recent audit, pending database count; UI фильтрует по дате, статусу, сканам, SkladBot, database.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -13782,7 +13106,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Scan валидирует код, блокирует КИЗ PostgreSQL advisory lock, проверяет дубль/другой заказ/SKU/aggregate box, пишет scan_codes, kiz_movements, audit и очередь Google export. Undo пишет movement undo, удаляет scan, пересчитывает blocks.</t>
+          <t>Scan валидирует код, блокирует КИЗ PostgreSQL advisory lock, проверяет дубль/другой заказ/SKU/aggregate box, пишет scan_codes, kiz_movements, audit и очередь database event. Undo пишет movement undo, удаляет scan, пересчитывает blocks.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -13834,7 +13158,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Complete требует все required blocks и повторный complete идемпотентен. Return ищет completed order, требует подтверждение всех позиций, пишет return movement, очередь SkladBot return и Google archive/returns exports.</t>
+          <t>Complete требует все required blocks и повторный complete идемпотентен. Return ищет completed order, требует подтверждение всех позиций, пишет return movement, очередь SkladBot return и backend completion/returns exports.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -13886,7 +13210,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/imports создает ImportJob, группирует orders/items, дедупит по source/import keys, backfill адресов, создает incident при ошибках, ставит Google import export и SkladBot dry-run.</t>
+          <t>/api/v1/imports создает ImportJob, группирует orders/items, дедупит по source/import keys, backfill адресов, создает incident при ошибках, ставит database import export и SkladBot dry-run.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -13938,7 +13262,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>UI требует выбор, reason, confirm, expected updated_at; backend повторно проверяет активность, сканы, pending Google, idempotency, audit и queue exports.</t>
+          <t>UI требует выбор, reason, confirm, expected updated_at; backend повторно проверяет активность, сканы, pending database, idempotency, audit и queue exports.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -14126,27 +13450,27 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Backend / Google</t>
+          <t>Backend / Database</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Google mirror sync/pending</t>
+          <t>DB-only runtime and XLSX interchange</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>live Google Sheets credentials/quota</t>
+          <t>live PostgreSQL credentials/quota</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Run against configured Google Sheets mirror with safe test order and verify pending/export/sync result.</t>
+          <t>Run against configured PostgreSQL mirror with safe test order and verify pending/export/sync result.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Pending exports идемпотентны; batch scan/archive; rate limit ставит pause. Google-to-backend sync обновляет поля, но не удаляет backend item при пропаже строки и игнорирует ручной Google return marker без backend return.</t>
+          <t>Pending exports идемпотентны; batch scan/archive; rate limit ставит pause. database-to-backend sync обновляет поля, но не удаляет backend item при пропаже строки и игнорирует ручной backend return marker без backend return.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -14198,7 +13522,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Import строит dry-run; default mode dry_run, enabled ставит create events; unknown SKU/zero qty блокирует; already linked не дублируется; stock shortage может удалить unscanned active order и queued Google cleanup.</t>
+          <t>Import строит dry-run; default mode dry_run, enabled ставит create events; unknown SKU/zero qty блокирует; already linked не дублируется; stock shortage может удалить unscanned active order и queued database cleanup.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -14250,7 +13574,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>DB source, Google mirror сравнивается по source keys, статусам/WH-R/dedup; Google down дает mirror_issue, не ломает DB workflow; критичные drift/SkladBot gaps создают incidents и Telegram notification events.</t>
+          <t>DB source, database state сравнивается по source keys, статусам/WH-R/dedup; database unavailable дает mirror_issue, не ломает DB workflow; критичные drift/SkladBot gaps создают incidents и Telegram notification events.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -14354,7 +13678,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Compose поднимает Postgres, backend, frontend, SkladBot worker, Google sync worker, Telegram worker, Adminer behind Traefik. Backup/restore через pg_dump/psql; acceptance проверяет health/ready/compose/verifiers.</t>
+          <t>Compose поднимает Postgres, backend, frontend, SkladBot worker, database sync worker, Telegram worker, Adminer behind Traefik. Backup/restore через pg_dump/psql; acceptance проверяет health/ready/compose/verifiers.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -14614,7 +13938,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Матчит по дате, клиенту, оплате, товарам/блокам; пишет found/multiple/not_found/pending; очередь Google export создается после обновления.</t>
+          <t>Матчит по дате, клиенту, оплате, товарам/блокам; пишет found/multiple/not_found/pending; очередь database event создается после обновления.</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -14807,12 +14131,12 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Postgres vs Google/SkladBot</t>
+          <t>Postgres vs database/SkladBot</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>live Telegram bot/chat permissions; live Google Sheets credentials/quota; live SkladBot API/tokens</t>
+          <t>live Telegram bot/chat permissions; live PostgreSQL credentials/quota; live SkladBot API/tokens</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -14822,7 +14146,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Postgres source of truth; сравнивает Google rows по source keys, статусы и WH-R; агрегирует SkladBot gaps; создает incidents и критичные Telegram alerts.</t>
+          <t>Postgres source of truth; сравнивает database rows по source keys, статусы и WH-R; агрегирует SkladBot gaps; создает incidents и критичные Telegram alerts.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -14945,162 +14269,6 @@
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-02 16:52 Asia/Tashkent</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-001</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Google Sheets</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Backend-to-Google exporter</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>Run against configured Google Sheets mirror with safe test order and verify pending/export/sync result.</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>Создает/обновляет layout, append/restore/delete rows, пишет сканы/status/SkladBot fields, переносит archive/cancel/no-KIZ/returns, сохраняет старый WH-R при pending.</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>accepted</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
-        </is>
-      </c>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
-        </is>
-      </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-02 16:52 Asia/Tashkent</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-002</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>Google Sheets</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Pending export retry</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>Run against configured Google Sheets mirror with safe test order and verify pending/export/sync result.</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>PendingEvent идемпотентен; scan/archive батчатся; rate limit оставляет события pending с next_attempt_at; stale processing сбрасывается.</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>accepted</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
-        </is>
-      </c>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
-        </is>
-      </c>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-02 16:52 Asia/Tashkent</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-003</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Google Sheets</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Google-to-backend sync</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Run against configured Google Sheets mirror with safe test order and verify pending/export/sync result.</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Матчит по source IDs, обновляет поля, не затирает SkladBot stale mirror, импортирует КИЗы через movement checks, конфликты логирует вместо удаления DB truth.</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>accepted</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
         <is>
           <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>

</xml_diff>

<commit_message>
feat: PostgreSQL-only runtime and return KIZ fix (#23)
* feat: decommission Google Sheets runtime

* fix: gate DB-only cutover on legacy data audit

* test: account for signing dependency SBOM
</commit_message>
<xml_diff>
--- a/docs/taksklad-feature-user-stories.xlsx
+++ b/docs/taksklad-feature-user-stories.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="User Stories" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Test Loop" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Errors" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Sources" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Manual Acceptance" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Stories" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Loop" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual Acceptance" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$22</definedName>
@@ -605,7 +605,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Still required for UI, Windows printer/updater, live Telegram, Google, SkladBot and VDS paths</t>
+          <t>Still required for UI, Windows printer/updater, live Telegram, database, SkladBot and VDS paths</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Automated portions continue to improve; manual/live acceptance remains pending for Windows UI, printer, updater, Telegram, Google, SkladBot and VDS dependent stories.</t>
+          <t>Automated portions continue to improve; manual/live acceptance remains pending for Windows UI, printer, updater, Telegram, database, SkladBot and VDS dependent stories.</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>ERR-004 false reconciliation mismatch; ERR-005 order-list search summary UX; ERR-006 reconciliation UTC default date; ERR-008 feature acceptance CLI gate; GAP-027/GAP-044 logistics no/invalid coordinates XLSX problem sheet; GAP-014/GAP-022 backend source-of-truth returns; GAP-046 PostgreSQL Google export row-lock contract; GAP-031 SQL/Alembic migration contract; GAP-024 web delete-active action; ERR-001 project .venv rebuilt to Python 3.12.13</t>
+          <t>ERR-004 false reconciliation mismatch; ERR-005 order-list search summary UX; ERR-006 reconciliation UTC default date; ERR-008 feature acceptance CLI gate; GAP-027/GAP-044 logistics no/invalid coordinates XLSX problem sheet; GAP-014/GAP-022 backend source-of-truth returns; GAP-046 PostgreSQL database event row-lock contract; GAP-031 SQL/Alembic migration contract; GAP-024 web delete-active action; ERR-001 project .venv rebuilt to Python 3.12.13</t>
         </is>
       </c>
     </row>
@@ -823,7 +823,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V48"/>
+  <dimension ref="A1:V45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -984,7 +984,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Entry points вызывают run_app для обычного запуска; --smoke-import проверяет импорт; --smoke-gui строит Tkinter UI, flushes layout и закрывает окно без mainloop/Google/backend данных; Windows release workflow запускает --smoke-import и --smoke-gui для onefile и onedir из clean temp dirs; без Google credentials и без backend-read обычный запуск показывает startup error.</t>
+          <t>Entry points вызывают run_app для обычного запуска; --smoke-import проверяет импорт; --smoke-gui строит Tkinter UI, flushes layout и закрывает окно без mainloop/database/backend данных; Windows release workflow запускает --smoke-import и --smoke-gui для onefile и onedir из clean temp dirs; без database credentials и без backend-read обычный запуск показывает startup error.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Backend read mode использует backend как primary; при падении backend идет Google fallback; SkladBot error не скрывает Google-заказы; текущая позиция сохраняется при refresh.</t>
+          <t>Backend read mode использует backend как primary; при падении backend идет legacy fallback; SkladBot error не скрывает database-заказы; текущая позиция сохраняется при refresh.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1538,12 +1538,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>src/taksklad/app_scanning.py; src/taksklad/scan_quantities.py; src/taksklad/desktop_scan_rules.py; tests/test_scan_quantities.py; tests/test_google_sheets_desktop_read.py; tests/test_desktop_ui_contract.py</t>
+          <t>src/taksklad/app_scanning.py; src/taksklad/scan_quantities.py; src/taksklad/desktop_scan_rules.py; tests/test_scan_quantities.py; tests/test_desktop_db_only_contract.py; tests/test_desktop_ui_contract.py</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_scan_quantities tests.test_google_sheets_desktop_read tests.test_desktop_ui_contract</t>
+          <t>python -m unittest tests.test_scan_quantities tests.test_desktop_db_only_contract tests.test_desktop_ui_contract</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Undo пишет backup, обновляет pending save/backend/Google, может очистить active row через allow_empty=True, блокирует finish если позиция стала неполной; archive/return/closed не откатывает.</t>
+          <t>Undo пишет backup, обновляет pending save/backend/database, может очистить active row через allow_empty=True, блокирует finish если позиция стала неполной; archive/return/closed не откатывает.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1866,12 +1866,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>src/taksklad/app_scanning.py; src/taksklad/pending_store.py; tests/test_desktop_pending_store.py; tests/test_desktop_ui_contract.py</t>
+          <t>src/taksklad/app_scanning.py; src/taksklad/pending_store.py; tests/test_desktop_db_only_contract.py; tests/test_desktop_ui_contract.py</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_pending_store tests.test_desktop_ui_contract tests.test_backend_bridge</t>
+          <t>python -m unittest tests.test_desktop_db_only_contract tests.test_desktop_ui_contract tests.test_backend_bridge</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Локальный/pending откат сохраненного кода покрыт и исправлен: saved_codes_count теперь уменьшается без Google/backend. Откат уже синхронизированного кода без pending-записи всё ещё требует доступного backend или Google и ручной Windows validation.</t>
+          <t>Локальный/pending откат сохраненного кода покрыт и исправлен: saved_codes_count теперь уменьшается без database/backend. Откат уже синхронизированного кода без pending-записи всё ещё требует доступного backend или database и ручной Windows validation.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>Run manual Windows acceptance for already-synced undo via live backend/Google; keep local pending-save regression green.</t>
+          <t>Run manual Windows acceptance for already-synced undo via live backend/database; keep local pending-save regression green.</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>DESK-09 pending-save/rollback regressions passed; desktop/backend undo subset 58 tests OK; full unittest discover 545 OK; py_compile OK. Local pending-save undo keeps saved_codes_count consistent without Google/backend; backend/Google live failure paths restore local state. Saved already-synced undo without pending record still needs live backend/Google + Windows acceptance.</t>
+          <t>DESK-09 pending-save/rollback regressions passed; desktop/backend undo subset 58 tests OK; full unittest discover 545 OK; py_compile OK. Local pending-save undo keeps saved_codes_count consistent without database/backend; backend/database live failure paths restore local state. Saved already-synced undo without pending record still needs live backend/database + Windows acceptance.</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>.venv/bin/python -m unittest tests.test_desktop_pending_store tests.test_desktop_ui_contract tests.test_backend_bridge; full unittest discover 545 OK; py_compile OK.</t>
+          <t>.venv/bin/python -m unittest tests.test_desktop_db_only_contract tests.test_desktop_ui_contract tests.test_backend_bridge; full unittest discover 545 OK; py_compile OK.</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>next_product требует exact plan, сохраняет в backend или Google, retryable Google error кладет pending save, пишет backup, последняя позиция ведет к ЗАВЕРШИТЬ ЗАКАЗ.</t>
+          <t>next_product требует exact plan, сохраняет в backend или database, retryable database error кладет pending save, пишет backup, последняя позиция ведет к ЗАВЕРШИТЬ ЗАКАЗ.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract tests.test_desktop_pending_store tests.test_backend_bridge</t>
+          <t>python -m unittest tests.test_desktop_ui_contract tests.test_desktop_db_only_contract tests.test_backend_bridge</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="V11" s="2" t="inlineStr">
         <is>
-          <t>.venv/bin/python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_next_product_hard_error_keeps_final_position_actions_consistent tests.test_desktop_ui_contract tests.test_desktop_pending_store tests.test_backend_bridge; full unittest discover 546 OK; py_compile OK.</t>
+          <t>.venv/bin/python -m unittest tests.test_desktop_db_only_contract tests.test_desktop_ui_contract tests.test_desktop_db_only_contract tests.test_backend_bridge; full unittest discover 546 OK; py_compile OK.</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2080,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Finish требует все позиции saved/full scanned; подтверждает параметры печати; add_pending_print создается до печати; backend complete/Google archive только после успешной печати.</t>
+          <t>Finish требует все позиции saved/full scanned; подтверждает параметры печати; add_pending_print создается до печати; backend complete/backend completion только после успешной печати.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Локальный риск очереди печати исправлен: finish/manual retry теперь проверяют успешную запись pending_print до печати и успешное удаление после печати до backend complete/Google archive. Физическая печать на Windows с реальным драйвером всё ещё требует validation.</t>
+          <t>Локальный риск очереди печати исправлен: finish/manual retry теперь проверяют успешную запись pending_print до печати и успешное удаление после печати до backend complete/backend completion. Физическая печать на Windows с реальным драйвером всё ещё требует validation.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>DESK-11 pending print queue regression: 60 tests OK; py_compile OK. Finish now requires confirmed pending_print add before print and confirmed pending_print remove before backend complete/Google archive. Manual physical Windows print validation remains pending.</t>
+          <t>DESK-11 pending print queue regression: 60 tests OK; py_compile OK. Finish now requires confirmed pending_print add before print and confirmed pending_print remove before backend complete/backend completion. Manual physical Windows print validation remains pending.</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>DESK-11 pending print queue regression: 60 tests OK; py_compile OK. Finish now requires confirmed pending_print add before print and confirmed pending_print remove before backend complete/Google archive. Manual physical Windows print validation remains pending.</t>
+          <t>DESK-11 pending print queue regression: 60 tests OK; py_compile OK. Finish now requires confirmed pending_print add before print and confirmed pending_print remove before backend complete/backend completion. Manual physical Windows print validation remains pending.</t>
         </is>
       </c>
     </row>
@@ -2314,12 +2314,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>src/taksklad/app_imports.py; src/taksklad/excel_import.py; tests/test_excel_import_append.py</t>
+          <t>src/taksklad/app_imports.py; src/taksklad/excel_import.py; tests/test_desktop_db_only_contract.py</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/Google commit remain pending.</t>
+          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/database commit remain pending.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Локально исправлены unsupported extension UX, backend-mode preview дублей/invalid rows и потеря координат desktop parser -&gt; backend. Остается ручная validation: полный Tkinter e2e на Windows, live Yandex geocoder, backend/Google commit на тестовом файле и визуальный preview.</t>
+          <t>Локально исправлены unsupported extension UX, backend-mode preview дублей/invalid rows и потеря координат desktop parser -&gt; backend. Остается ручная validation: полный Tkinter e2e на Windows, live Yandex geocoder, backend/database commit на тестовом файле и визуальный preview.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>Run manual Windows acceptance: choose .xlsx/.xlsm, verify preview counts for new/duplicate/invalid rows, confirm backend import, check active orders/logistics coordinates, legacy Google fallback, unsupported file warning, and live geocoding.</t>
+          <t>Run manual Windows acceptance: choose .xlsx/.xlsm, verify preview counts for new/duplicate/invalid rows, confirm backend import, check active orders/logistics coordinates, legacy legacy fallback, unsupported file warning, and live geocoding.</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="T14" s="2" t="inlineStr">
         <is>
-          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/Google commit remain pending.</t>
+          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/database commit remain pending.</t>
         </is>
       </c>
       <c r="U14" s="2" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="V14" s="2" t="inlineStr">
         <is>
-          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/Google commit remain pending.</t>
+          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/database commit remain pending.</t>
         </is>
       </c>
     </row>
@@ -2416,7 +2416,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Окно ищет заявку, показывает состав, требует confirmed_items; backend mode читает/пишет backend; Google-only возврат без _backend_order_id отклоняется; legacy Google fallback сохранен только вне backend mode.</t>
+          <t>Окно ищет заявку, показывает состав, требует confirmed_items; backend mode читает/пишет backend; legacy-only возврат без _backend_order_id отклоняется; legacy legacy fallback сохранен только вне backend mode.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_google_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects</t>
+          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_legacy_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Manual Windows return UI acceptance remains pending; local legacy Google totals display fixed and retested.</t>
+          <t>Manual Windows return UI acceptance remains pending; local legacy database totals display fixed and retested.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>Run manual Windows returns acceptance: lookup, confirmation dialog, backend return, returned list, legacy Google fallback only when backend mode is off.</t>
+          <t>Run manual Windows returns acceptance: lookup, confirmation dialog, backend return, returned list, legacy legacy fallback only when backend mode is off.</t>
         </is>
       </c>
       <c r="Q15" s="2" t="inlineStr">
@@ -2486,17 +2486,17 @@
       </c>
       <c r="T15" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_google_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects - 13 tests OK; python -m py_compile src/taksklad/app_returns.py tests/test_desktop_ui_contract.py backend/app/orders_service.py tests/test_backend_api_persistence.py - OK.</t>
+          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_legacy_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects - 13 tests OK; python -m py_compile src/taksklad/app_returns.py tests/test_desktop_ui_contract.py backend/app/orders_service.py tests/test_backend_api_persistence.py - OK.</t>
         </is>
       </c>
       <c r="U15" s="2" t="inlineStr">
         <is>
-          <t>GAP-014 fixed_retested: desktop return path sends confirmed_items to backend, does not use Google fallback in backend mode, and return totals now correctly display both backend and legacy Google item shapes.</t>
+          <t>GAP-014 fixed_retested: desktop return path sends confirmed_items to backend, does not use legacy fallback in backend mode, and return totals now correctly display both backend and legacy database item shapes.</t>
         </is>
       </c>
       <c r="V15" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_google_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects - 13 tests OK; python -m py_compile src/taksklad/app_returns.py tests/test_desktop_ui_contract.py backend/app/orders_service.py tests/test_backend_api_persistence.py - OK.</t>
+          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_legacy_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects - 13 tests OK; python -m py_compile src/taksklad/app_returns.py tests/test_desktop_ui_contract.py backend/app/orders_service.py tests/test_backend_api_persistence.py - OK.</t>
         </is>
       </c>
     </row>
@@ -3079,12 +3079,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Как админ склада, хочу видеть все позиции, статусы, суммы, Google/SkladBot/return state.</t>
+          <t>Как админ склада, хочу видеть все позиции, статусы, суммы, database/SkladBot/return state.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/admin/table строит плоские строки по позициям, totals по всем строкам, recent audit, pending Google count; endpoint поддерживает limit/offset и page metadata; UI показывает загружено/всего, фильтрует загруженные строки и дает догрузить следующую страницу.</t>
+          <t>/api/v1/admin/table строит плоские строки по позициям, totals по всем строкам, recent audit, pending database count; endpoint поддерживает limit/offset и page metadata; UI показывает загружено/всего, фильтрует загруженные строки и дает догрузить следующую страницу.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -3192,7 +3192,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Scan валидирует код, блокирует КИЗ PostgreSQL advisory lock, проверяет дубль/другой заказ/SKU/aggregate box, пишет scan_codes, kiz_movements, audit и очередь Google export. Undo пишет movement undo, удаляет scan, пересчитывает blocks.</t>
+          <t>Scan валидирует код, блокирует КИЗ PostgreSQL advisory lock, проверяет дубль/другой заказ/SKU/aggregate box, пишет scan_codes, kiz_movements, audit и очередь database event. Undo пишет movement undo, удаляет scan, пересчитывает blocks.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -3202,12 +3202,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>backend/app/orders_service.py; backend/app/google_sheets_pending.py; backend/app/kiz_movements_service.py; backend/app/schemas.py; tests/test_backend_api_persistence.py; tests/test_backend_google_sheets_pending.py</t>
+          <t>backend/app/orders_service.py; backend/app/event_queue_service.py; backend/app/kiz_movements_service.py; backend/app/schemas.py; tests/test_backend_api_persistence.py; tests/test_backend_db_only_runtime.py</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_backend_api_persistence tests.test_backend_google_sheets_pending</t>
+          <t>python -m unittest tests.test_backend_api_persistence tests.test_backend_db_only_runtime</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Local/API scan and Google export queue lock covered; operator/UI/live acceptance remains pending.</t>
+          <t>Local/API scan and database event queue lock covered; operator/UI/live acceptance remains pending.</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -3262,7 +3262,7 @@
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_google_sheets_export_when_google_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_google_sheets_best_effort OK; py_compile backend/app/google_sheets_pending.py tests/test_backend_google_sheets_pending.py tests/test_backend_api_persistence.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_database_export_when_database_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_database_best_effort OK; py_compile backend/app/event_queue_service.py tests/test_backend_db_only_runtime.py tests/test_backend_api_persistence.py OK.</t>
         </is>
       </c>
       <c r="U22" s="2" t="inlineStr">
@@ -3272,7 +3272,7 @@
       </c>
       <c r="V22" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_google_sheets_export_when_google_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_google_sheets_best_effort OK; py_compile backend/app/google_sheets_pending.py tests/test_backend_google_sheets_pending.py tests/test_backend_api_persistence.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_database_export_when_database_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_database_best_effort OK; py_compile backend/app/event_queue_service.py tests/test_backend_db_only_runtime.py tests/test_backend_api_persistence.py OK.</t>
         </is>
       </c>
     </row>
@@ -3304,7 +3304,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Complete требует все required blocks и повторный complete идемпотентен. Return ищет completed order, требует подтверждение всех позиций, пишет return movement, очередь SkladBot return и Google archive/returns exports; Google mirror не source of truth.</t>
+          <t>Complete требует все required blocks и повторный complete идемпотентен. Return ищет completed order, требует подтверждение всех позиций, пишет return movement, очередь SkladBot return и backend completion/returns exports; database state не source of truth.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -3370,17 +3370,17 @@
       </c>
       <c r="T23" s="2" t="inlineStr">
         <is>
-          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items - 12 tests OK</t>
+          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items - 12 tests OK</t>
         </is>
       </c>
       <c r="U23" s="2" t="inlineStr">
         <is>
-          <t>GAP-022 fixed_retested: backend returns are source of truth; Google is best-effort mirror/export.</t>
+          <t>GAP-022 fixed_retested: backend returns are source of truth; database is best-effort mirror/export.</t>
         </is>
       </c>
       <c r="V23" s="2" t="inlineStr">
         <is>
-          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items - 12 tests OK</t>
+          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items - 12 tests OK</t>
         </is>
       </c>
     </row>
@@ -3412,7 +3412,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/imports создает ImportJob, группирует orders/items, дедупит по source/import keys, backfill адресов, создает incident при ошибках, ставит Google import export и SkladBot dry-run.</t>
+          <t>/api/v1/imports создает ImportJob, группирует orders/items, дедупит по source/import keys, backfill адресов, создает incident при ошибках, ставит database import export и SkladBot dry-run.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -3422,7 +3422,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>backend/app/imports_service.py; backend/app/google_sheets_pending.py; backend/app/schemas.py; tests/test_backend_api_persistence.py</t>
+          <t>backend/app/imports_service.py; backend/app/event_queue_service.py; backend/app/schemas.py; tests/test_backend_api_persistence.py</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -3442,7 +3442,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>Postgres import survives Google export queue failure and records incident/audit; operator/live acceptance remains pending.</t>
+          <t>Postgres import survives database event queue failure and records incident/audit; operator/live acceptance remains pending.</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="T24" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_google_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_google_sheets_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_google_sheets tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write OK; py_compile backend/app/imports_service.py tests/test_backend_api_persistence.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_database_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_database_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_database tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write OK; py_compile backend/app/imports_service.py tests/test_backend_api_persistence.py OK.</t>
         </is>
       </c>
       <c r="U24" s="2" t="inlineStr">
@@ -3492,7 +3492,7 @@
       </c>
       <c r="V24" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_google_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_google_sheets_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_google_sheets tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write OK; py_compile backend/app/imports_service.py tests/test_backend_api_persistence.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_database_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_database_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_database tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write OK; py_compile backend/app/imports_service.py tests/test_backend_api_persistence.py OK.</t>
         </is>
       </c>
     </row>
@@ -3519,12 +3519,12 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Как админ, хочу безопасно архивировать, отменять, reset/rescan, restore, resync Google/SkladBot и bulk complete без КИЗ.</t>
+          <t>Как админ, хочу безопасно архивировать, отменять, reset/rescan, restore, resync database/SkladBot и bulk complete без КИЗ.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>UI требует выбор, reason, confirm, expected updated_at; backend повторно проверяет активность, сканы, pending Google, idempotency, audit и queue exports.</t>
+          <t>UI требует выбор, reason, confirm, expected updated_at; backend повторно проверяет активность, сканы, pending database, idempotency, audit и queue exports.</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -3944,12 +3944,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Backend / Google</t>
+          <t>Backend / Database</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Google mirror sync/pending</t>
+          <t>DB-only runtime and XLSX interchange</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -3959,12 +3959,12 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Как оператор, хочу, чтобы Postgres оставался source of truth, а Google синхронизировался надежно.</t>
+          <t>Как оператор, хочу, чтобы Postgres оставался source of truth, а database синхронизировался надежно.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Pending exports идемпотентны; batch scan/archive; rate limit ставит pause. Google-to-backend sync обновляет поля, но не удаляет backend item при пропаже строки и игнорирует ручной Google return marker без backend return.</t>
+          <t>PostgreSQL is the only runtime source of truth; XLSX is used only for preview, import and export; no spreadsheet credentials, workers or fallback paths are required.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -3974,12 +3974,12 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>backend/app/google_sheets_pending.py; backend/app/google_sheets_sync_worker.py; backend/app/reconciliation_service.py; tests/test_backend_google_sheets_pending.py; tests/test_google_sheets_sync_worker.py; tests/test_reconciliation_service.py</t>
+          <t>backend/app/excel_web_service.py; backend/app/admin_orders_export_service.py; backend/app/event_queue_service.py; tests/test_backend_db_only_runtime.py; tests/test_google_sheets_decommission_contract.py</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_backend_google_sheets_pending tests.test_google_sheets_sync_worker tests.test_reconciliation_service</t>
+          <t>python -m unittest tests.test_backend_db_only_runtime tests.test_backend_db_only_runtime tests.test_reconciliation_service</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -3994,7 +3994,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>Google 429 retry cooldown is enforced locally; mirror drift is covered by reconciliation flow. Live Google credentials/quota acceptance remains pending.</t>
+          <t>database 429 retry cooldown is enforced locally; mirror drift is covered by reconciliation flow. Live database credentials/quota acceptance remains pending.</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
@@ -4029,12 +4029,12 @@
       </c>
       <c r="S29" s="2" t="inlineStr">
         <is>
-          <t>live Google Sheets credentials/quota</t>
+          <t>live PostgreSQL credentials/quota</t>
         </is>
       </c>
       <c r="T29" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event OK; py_compile backend/app/google_sheets_pending.py tests/test_backend_google_sheets_pending.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event OK; py_compile backend/app/event_queue_service.py tests/test_backend_db_only_runtime.py OK.</t>
         </is>
       </c>
       <c r="U29" s="2" t="inlineStr">
@@ -4044,7 +4044,7 @@
       </c>
       <c r="V29" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event OK; py_compile backend/app/google_sheets_pending.py tests/test_backend_google_sheets_pending.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event OK; py_compile backend/app/event_queue_service.py tests/test_backend_db_only_runtime.py OK.</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Import строит dry-run; default mode dry_run, enabled ставит create events; unknown SKU/zero qty блокирует; already linked не дублируется; stock shortage может удалить unscanned active order и queued Google cleanup.</t>
+          <t>Import строит dry-run; default mode dry_run, enabled ставит create events; unknown SKU/zero qty блокирует; already linked не дублируется; stock shortage может удалить unscanned active order и queued database cleanup.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -4183,12 +4183,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Как ответственный, хочу видеть расхождения DB vs Google/SkladBot и получать alerts.</t>
+          <t>Как ответственный, хочу видеть расхождения DB vs database/SkladBot и получать alerts.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>DB source, Google mirror сравнивается по source keys, статусам/WH-R/dedup; Google down дает mirror_issue, не ломает DB workflow; критичные drift/SkladBot gaps создают incidents и Telegram notification events.</t>
+          <t>DB source, database state сравнивается по source keys, статусам/WH-R/dedup; database unavailable дает mirror_issue, не ломает DB workflow; критичные drift/SkladBot gaps создают incidents и Telegram notification events.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -4218,7 +4218,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Returned DB status может легитимно соответствовать Google Выполнено; риск регрессии высокий.</t>
+          <t>Returned DB status может легитимно соответствовать database Выполнено; риск регрессии высокий.</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Compose поднимает Postgres, backend, frontend, SkladBot worker, Google sync worker, Telegram worker, Adminer behind Traefik. Backup/restore через pg_dump/psql; acceptance проверяет health/ready/compose/verifiers.</t>
+          <t>Compose поднимает Postgres, backend, frontend, SkladBot worker, database sync worker, Telegram worker, Adminer behind Traefik. Backup/restore через pg_dump/psql; acceptance проверяет health/ready/compose/verifiers.</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Матчит по дате, клиенту, оплате, товарам/блокам; пишет found/multiple/not_found/pending; очередь Google export создается после обновления.</t>
+          <t>Матчит по дате, клиенту, оплате, товарам/блокам; пишет found/multiple/not_found/pending; очередь database event создается после обновления.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -5353,7 +5353,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Postgres vs Google/SkladBot</t>
+          <t>Postgres vs database/SkladBot</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -5368,7 +5368,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Postgres source of truth; сравнивает Google rows по source keys, статусы и WH-R; агрегирует SkladBot gaps; создает incidents и критичные Telegram alerts.</t>
+          <t>Postgres source of truth; сравнивает database rows по source keys, статусы и WH-R; агрегирует SkladBot gaps; создает incidents и критичные Telegram alerts.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -5398,7 +5398,7 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>API endpoint сам не шлет alerts; при недоступном Google статус mirror_issue без деталей mismatch.</t>
+          <t>API endpoint сам не шлет alerts; при недоступном database статус mirror_issue без деталей mismatch.</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr">
@@ -5433,7 +5433,7 @@
       </c>
       <c r="S42" s="2" t="inlineStr">
         <is>
-          <t>live Telegram bot/chat permissions; live Google Sheets credentials/quota; live SkladBot API/tokens</t>
+          <t>live Telegram bot/chat permissions; live PostgreSQL credentials/quota; live SkladBot API/tokens</t>
         </is>
       </c>
       <c r="T42" s="2" t="inlineStr">
@@ -5783,322 +5783,6 @@
           <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_logistics_report_uses_shipment_date_coordinates_and_prices tests.test_backend_api_persistence.BackendApiPersistenceTests.test_logistics_report_keeps_unrouteable_orders_on_separate_sheet tests.test_backend_api_persistence.BackendApiPersistenceTests.test_logistics_report_returns_unrouteable_sheet_when_date_has_no_routeable_orders tests.test_backend_api_persistence.BackendApiPersistenceTests.test_logistics_report_404_when_date_has_only_pickup_orders tests.test_backend_api_persistence.BackendApiPersistenceTests.test_logistics_report_normalizes_three_part_coordinates tests.test_backend_skladbot_request_dry_run.BackendSkladBotRequestDryRunTests.test_logistics_report_excludes_stock_shortage_blocked_order - 6 tests OK</t>
         </is>
       </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-001</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Google Sheets</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Backend-to-Google exporter</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Как backend, я синхронизирую Google-зеркало без дублей.</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Создает/обновляет layout, append/restore/delete rows, пишет сканы/status/SkladBot fields, переносит archive/cancel/no-KIZ/returns, сохраняет старый WH-R при pending.</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>Code/docs/tests</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/google_sheets_exporter.py; tests/test_backend_google_sheets_exporter.py</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_backend_google_sheets_exporter</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>covered_auto_manual_pending</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>manual_required</t>
-        </is>
-      </c>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>При credentials выполняет реальные Google writes; без них действия должны ретраиться через очередь.</t>
-        </is>
-      </c>
-      <c r="M46" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="N46" s="2" t="inlineStr">
-        <is>
-          <t>auto+manual</t>
-        </is>
-      </c>
-      <c r="O46" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 13:31 Asia/Tashkent</t>
-        </is>
-      </c>
-      <c r="P46" s="2" t="inlineStr">
-        <is>
-          <t>Run manual acceptance for UI/integration/hardware parts</t>
-        </is>
-      </c>
-      <c r="Q46" s="2" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="R46" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="S46" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="T46" s="2" t="inlineStr">
-        <is>
-          <t>Full verifier: unittest discover 531 OK; py_compile OK; frontend build OK; compose/shell/audit/preflight/diff OK. Feature gate status OK but manual/open-error gates intentionally red.</t>
-        </is>
-      </c>
-      <c r="U46" s="2" t="n"/>
-      <c r="V46" s="2" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-002</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>Google Sheets</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Pending export retry</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>Оператор/система</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>Как оператор, я хочу безопасный retry Google-операций.</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>PendingEvent идемпотентен; scan/archive батчатся; PostgreSQL claim использует FOR UPDATE SKIP LOCKED вместо session advisory lock; rate limit оставляет события pending с next_attempt_at; stale processing сбрасывается.</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>Code/docs/tests</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/google_sheets_pending.py; tests/test_backend_google_sheets_pending.py</t>
-        </is>
-      </c>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_backend_google_sheets_pending</t>
-        </is>
-      </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>covered_auto_manual_pending</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="inlineStr">
-        <is>
-          <t>manual_required</t>
-        </is>
-      </c>
-      <c r="L47" s="2" t="n"/>
-      <c r="M47" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="N47" s="2" t="inlineStr">
-        <is>
-          <t>auto+manual</t>
-        </is>
-      </c>
-      <c r="O47" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 13:47 Asia/Tashkent</t>
-        </is>
-      </c>
-      <c r="P47" s="2" t="inlineStr">
-        <is>
-          <t>Run manual acceptance for UI/integration/hardware parts</t>
-        </is>
-      </c>
-      <c r="Q47" s="2" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="R47" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="S47" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="T47" s="2" t="inlineStr">
-        <is>
-          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_lock_does_not_use_session_level_advisory_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch - 3 tests OK</t>
-        </is>
-      </c>
-      <c r="U47" s="2" t="inlineStr">
-        <is>
-          <t>GAP-046 fixed_retested: PostgreSQL Google export queue is protected by row-level FOR UPDATE SKIP LOCKED, not session-level advisory lock.</t>
-        </is>
-      </c>
-      <c r="V47" s="2" t="inlineStr">
-        <is>
-          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_lock_does_not_use_session_level_advisory_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch - 3 tests OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-003</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Google Sheets</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Google-to-backend sync</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Оператор/система</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Как оператор, если включены ручные правки в Sheet, backend импортирует только безопасные изменения.</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>Матчит по source IDs, обновляет поля, не затирает SkladBot stale mirror, импортирует КИЗы через movement checks, конфликты логирует вместо удаления DB truth.</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>Code/docs/tests</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/google_sheets_sync_worker.py; tests/test_google_sheets_sync_worker.py</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_google_sheets_sync_worker</t>
-        </is>
-      </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>covered_auto_manual_pending</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>manual_required</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
-          <t>High-risk режим: Google может писать в Postgres; manual return columns игнорируются без backend return source.</t>
-        </is>
-      </c>
-      <c r="M48" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="N48" s="2" t="inlineStr">
-        <is>
-          <t>auto+manual</t>
-        </is>
-      </c>
-      <c r="O48" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 13:31 Asia/Tashkent</t>
-        </is>
-      </c>
-      <c r="P48" s="2" t="inlineStr">
-        <is>
-          <t>Run manual acceptance for UI/integration/hardware parts</t>
-        </is>
-      </c>
-      <c r="Q48" s="2" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="R48" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="S48" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="T48" s="2" t="inlineStr">
-        <is>
-          <t>Full verifier: unittest discover 531 OK; py_compile OK; frontend build OK; compose/shell/audit/preflight/diff OK. Feature gate status OK but manual/open-error gates intentionally red.</t>
-        </is>
-      </c>
-      <c r="U48" s="2" t="n"/>
-      <c r="V48" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:V48"/>
@@ -6120,7 +5804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N48"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6224,7 +5908,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Entry points вызывают run_app для обычного запуска; --smoke-import проверяет импорт; --smoke-gui строит Tkinter UI, flushes layout и закрывает окно без mainloop/Google/backend данных; Windows release workflow запускает --smoke-import и --smoke-gui для onefile и onedir из clean temp dirs; без Google credentials и без backend-read обычный запуск показывает startup error.</t>
+          <t>Entry points вызывают run_app для обычного запуска; --smoke-import проверяет импорт; --smoke-gui строит Tkinter UI, flushes layout и закрывает окно без mainloop/database/backend данных; Windows release workflow запускает --smoke-import и --smoke-gui для onefile и onedir из clean temp dirs; без database credentials и без backend-read обычный запуск показывает startup error.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -6360,7 +6044,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Backend read mode использует backend как primary; при падении backend идет Google fallback; SkladBot error не скрывает Google-заказы; текущая позиция сохраняется при refresh.</t>
+          <t>Backend read mode использует backend как primary; при падении backend идет legacy fallback; SkladBot error не скрывает database-заказы; текущая позиция сохраняется при refresh.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -6559,7 +6243,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_scan_quantities tests.test_google_sheets_desktop_read tests.test_desktop_ui_contract</t>
+          <t>python -m unittest tests.test_scan_quantities tests.test_desktop_db_only_contract tests.test_desktop_ui_contract</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -6580,7 +6264,7 @@
       <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>src/taksklad/app_scanning.py; src/taksklad/scan_quantities.py; src/taksklad/desktop_scan_rules.py; tests/test_scan_quantities.py; tests/test_google_sheets_desktop_read.py; tests/test_desktop_ui_contract.py</t>
+          <t>src/taksklad/app_scanning.py; src/taksklad/scan_quantities.py; src/taksklad/desktop_scan_rules.py; tests/test_scan_quantities.py; tests/test_desktop_db_only_contract.py; tests/test_desktop_ui_contract.py</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -6610,7 +6294,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_scan_quantities tests.test_google_sheets_desktop_read tests.test_desktop_ui_contract</t>
+          <t>python -m unittest tests.test_scan_quantities tests.test_desktop_db_only_contract tests.test_desktop_ui_contract</t>
         </is>
       </c>
     </row>
@@ -6763,17 +6447,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_pending_store tests.test_desktop_ui_contract tests.test_backend_bridge</t>
+          <t>python -m unittest tests.test_desktop_db_only_contract tests.test_desktop_ui_contract tests.test_backend_bridge</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Undo пишет backup, обновляет pending save/backend/Google, может очистить active row через allow_empty=True, блокирует finish если позиция стала неполной; archive/return/closed не откатывает.</t>
+          <t>Undo пишет backup, обновляет pending save/backend/database, может очистить active row через allow_empty=True, блокирует finish если позиция стала неполной; archive/return/closed не откатывает.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>DESK-09 pending-save/rollback regressions passed; desktop/backend undo subset 58 tests OK; full unittest discover 545 OK; py_compile OK. Local pending-save undo keeps saved_codes_count consistent without Google/backend; backend/Google live failure paths restore local state. Saved already-synced undo without pending record still needs live backend/Google + Windows acceptance.</t>
+          <t>DESK-09 pending-save/rollback regressions passed; desktop/backend undo subset 58 tests OK; full unittest discover 545 OK; py_compile OK. Local pending-save undo keeps saved_codes_count consistent without database/backend; backend/database live failure paths restore local state. Saved already-synced undo without pending record still needs live backend/database + Windows acceptance.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -6788,7 +6472,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>src/taksklad/app_scanning.py; src/taksklad/pending_store.py; src/taksklad/backend_events.py; tests/test_desktop_pending_store.py; tests/test_desktop_ui_contract.py; tests/test_backend_bridge.py</t>
+          <t>src/taksklad/app_scanning.py; src/taksklad/pending_store.py; src/taksklad/backend_events.py; tests/test_desktop_db_only_contract.py; tests/test_desktop_ui_contract.py; tests/test_backend_bridge.py</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -6813,12 +6497,12 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>DESK-09 pending-save/rollback regressions passed; desktop/backend undo subset 58 tests OK; full unittest discover 545 OK; py_compile OK. Local pending-save undo keeps saved_codes_count consistent without Google/backend; backend/Google live failure paths restore local state. Saved already-synced undo without pending record still needs live backend/Google + Windows acceptance.</t>
+          <t>DESK-09 pending-save/rollback regressions passed; desktop/backend undo subset 58 tests OK; full unittest discover 545 OK; py_compile OK. Local pending-save undo keeps saved_codes_count consistent without database/backend; backend/database live failure paths restore local state. Saved already-synced undo without pending record still needs live backend/database + Windows acceptance.</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>.venv/bin/python -m unittest tests.test_desktop_pending_store tests.test_desktop_ui_contract tests.test_backend_bridge</t>
+          <t>.venv/bin/python -m unittest tests.test_desktop_db_only_contract tests.test_desktop_ui_contract tests.test_backend_bridge</t>
         </is>
       </c>
     </row>
@@ -6835,12 +6519,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract tests.test_desktop_pending_store tests.test_backend_bridge</t>
+          <t>python -m unittest tests.test_desktop_ui_contract tests.test_desktop_db_only_contract tests.test_backend_bridge</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>next_product требует exact plan, сохраняет в backend или Google, retryable Google error кладет pending save, пишет backup, последняя позиция ведет к ЗАВЕРШИТЬ ЗАКАЗ.</t>
+          <t>next_product требует exact plan, сохраняет в backend или database, retryable database error кладет pending save, пишет backup, последняя позиция ведет к ЗАВЕРШИТЬ ЗАКАЗ.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -6860,7 +6544,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>src/taksklad/app_scanning.py; src/taksklad/app_finish.py; tests/test_desktop_ui_contract.py; tests/test_desktop_pending_store.py; tests/test_backend_bridge.py</t>
+          <t>src/taksklad/app_scanning.py; src/taksklad/app_finish.py; tests/test_desktop_ui_contract.py; tests/test_desktop_db_only_contract.py; tests/test_backend_bridge.py</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -6890,7 +6574,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>.venv/bin/python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_next_product_hard_error_keeps_final_position_actions_consistent tests.test_desktop_ui_contract tests.test_desktop_pending_store tests.test_backend_bridge</t>
+          <t>.venv/bin/python -m unittest tests.test_desktop_db_only_contract tests.test_desktop_ui_contract tests.test_desktop_db_only_contract tests.test_backend_bridge</t>
         </is>
       </c>
     </row>
@@ -6912,7 +6596,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Finish требует все позиции saved/full scanned; подтверждает параметры печати; add_pending_print создается до печати; backend complete/Google archive только после успешной печати.</t>
+          <t>Finish требует все позиции saved/full scanned; подтверждает параметры печати; add_pending_print создается до печати; backend complete/backend completion только после успешной печати.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -6953,7 +6637,7 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>DESK-11 pending print queue regression: 60 tests OK; py_compile OK. Finish now requires confirmed pending_print add before print and confirmed pending_print remove before backend complete/Google archive. Manual physical Windows print validation remains pending.</t>
+          <t>DESK-11 pending print queue regression: 60 tests OK; py_compile OK. Finish now requires confirmed pending_print add before print and confirmed pending_print remove before backend complete/backend completion. Manual physical Windows print validation remains pending.</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -7053,7 +6737,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/Google commit remain pending.</t>
+          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/database commit remain pending.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -7068,7 +6752,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/Google commit remain pending.</t>
+          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/database commit remain pending.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -7093,7 +6777,7 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/Google commit remain pending.</t>
+          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/database commit remain pending.</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -7115,17 +6799,17 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_google_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects</t>
+          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_legacy_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Окно ищет заявку, показывает состав, требует confirmed_items; backend mode читает/пишет backend; Google-only возврат без _backend_order_id отклоняется; legacy Google fallback сохранен только вне backend mode.</t>
+          <t>Окно ищет заявку, показывает состав, требует confirmed_items; backend mode читает/пишет backend; legacy-only возврат без _backend_order_id отклоняется; legacy legacy fallback сохранен только вне backend mode.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Desktop/backend return targeted tests OK: confirmed_items, backend-only list/lookup, Google-only rejection in backend mode, legacy fallback, KIZ release history, and backend/Google item totals display.</t>
+          <t>Desktop/backend return targeted tests OK: confirmed_items, backend-only list/lookup, legacy-only rejection in backend mode, legacy fallback, KIZ release history, and backend/database item totals display.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -7161,12 +6845,12 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_google_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects - 13 tests OK; python -m py_compile src/taksklad/app_returns.py tests/test_desktop_ui_contract.py backend/app/orders_service.py tests/test_backend_api_persistence.py - OK.</t>
+          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_legacy_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects - 13 tests OK; python -m py_compile src/taksklad/app_returns.py tests/test_desktop_ui_contract.py backend/app/orders_service.py tests/test_backend_api_persistence.py - OK.</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_google_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects</t>
+          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_legacy_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects</t>
         </is>
       </c>
     </row>
@@ -7591,17 +7275,17 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_backend_api_persistence tests.test_backend_google_sheets_pending</t>
+          <t>python -m unittest tests.test_backend_api_persistence tests.test_backend_db_only_runtime</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Scan валидирует код, блокирует КИЗ PostgreSQL advisory lock, проверяет дубль/другой заказ/SKU/aggregate box, пишет scan_codes, kiz_movements, audit и очередь Google export. Undo пишет movement undo, удаляет scan, пересчитывает blocks.</t>
+          <t>Scan валидирует код, блокирует КИЗ PostgreSQL advisory lock, проверяет дубль/другой заказ/SKU/aggregate box, пишет scan_codes, kiz_movements, audit и очередь database event. Undo пишет movement undo, удаляет scan, пересчитывает blocks.</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Scan best-effort Google queue is covered; non-Postgres Google export lock returns busy without processing; rate-limit leaves events pending. Manual/live acceptance still pending.</t>
+          <t>Scan best-effort database queue is covered; non-Postgres database event lock returns busy without processing; rate-limit leaves events pending. Manual/live acceptance still pending.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -7637,12 +7321,12 @@
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_google_sheets_export_when_google_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_google_sheets_best_effort OK; py_compile backend/app/google_sheets_pending.py tests/test_backend_google_sheets_pending.py tests/test_backend_api_persistence.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_database_export_when_database_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_database_best_effort OK; py_compile backend/app/event_queue_service.py tests/test_backend_db_only_runtime.py tests/test_backend_api_persistence.py OK.</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_google_sheets_export_when_google_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_google_sheets_best_effort tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch</t>
+          <t>python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_database_export_when_database_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_database_best_effort tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch</t>
         </is>
       </c>
     </row>
@@ -7664,12 +7348,12 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Complete требует все required blocks и повторный complete идемпотентен. Return ищет completed order, требует подтверждение всех позиций, пишет return movement, очередь SkladBot return и Google archive/returns exports; Google mirror не source of truth.</t>
+          <t>Complete требует все required blocks и повторный complete идемпотентен. Return ищет completed order, требует подтверждение всех позиций, пишет return movement, очередь SkladBot return и backend completion/returns exports; database state не source of truth.</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Backend return targeted tests OK: lookup/mark/list, duplicate guard, KIZ return/re_outbound movement, failed return no side effects, Google export best-effort, mismatch reject. Manual acceptance still pending.</t>
+          <t>Backend return targeted tests OK: lookup/mark/list, duplicate guard, KIZ return/re_outbound movement, failed return no side effects, database event best-effort, mismatch reject. Manual acceptance still pending.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -7705,7 +7389,7 @@
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items - 12 tests OK</t>
+          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items - 12 tests OK</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
@@ -7732,12 +7416,12 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/imports создает ImportJob, группирует orders/items, дедупит по source/import keys, backfill адресов, создает incident при ошибках, ставит Google import export и SkladBot dry-run.</t>
+          <t>/api/v1/imports создает ImportJob, группирует orders/items, дедупит по source/import keys, backfill адресов, создает incident при ошибках, ставит database import export и SkladBot dry-run.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Import creates Postgres order/items before Google export; Google queue storage failure returns 201 with google_sheets_status=error, keeps backend data, and creates incident/audit. Manual/live acceptance still pending.</t>
+          <t>Import creates Postgres order/items before database event; database queue storage failure returns 201 with database_status=error, keeps backend data, and creates incident/audit. Manual/live acceptance still pending.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -7773,12 +7457,12 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_google_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_google_sheets_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_google_sheets tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write OK; py_compile backend/app/imports_service.py tests/test_backend_api_persistence.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_database_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_database_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_database tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write OK; py_compile backend/app/imports_service.py tests/test_backend_api_persistence.py OK.</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_google_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_google_sheets_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_google_sheets tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write</t>
+          <t>python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_database_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_database_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_database tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write</t>
         </is>
       </c>
     </row>
@@ -7800,12 +7484,12 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>UI требует выбор, reason, confirm, expected updated_at; backend повторно проверяет активность, сканы, pending Google, idempotency, audit и queue exports.</t>
+          <t>UI требует выбор, reason, confirm, expected updated_at; backend повторно проверяет активность, сканы, pending database, idempotency, audit и queue exports.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Frontend web action bar exposes delete-active with reason/confirm and expected_updated_at payload; backend tests keep active/no-scan/pending Google/idempotency/audit/export preconditions. Manual browser smoke still pending.</t>
+          <t>Frontend web action bar exposes delete-active with reason/confirm and expected_updated_at payload; backend tests keep active/no-scan/pending database/idempotency/audit/export preconditions. Manual browser smoke still pending.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -7846,7 +7530,7 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>npm run build; tests.test_backend_api_persistence.BackendApiPersistenceTests.test_delete_active_order_removes_unscanned_order_and_queues_google_delete; tests.test_backend_api_persistence.BackendApiPersistenceTests.test_delete_active_order_idempotency_prevents_duplicate_audit_and_export; tests.test_backend_api_persistence.BackendApiPersistenceTests.test_delete_active_order_rejects_order_with_scans; tests.test_backend_telegram_import.BackendTelegramImportTests.test_telegram_worker_manual_delete_active_order_calls_safe_backend_endpoint; tests.test_backend_telegram_import.BackendTelegramImportTests.test_telegram_worker_manual_delete_refuses_started_order_before_backend_call</t>
+          <t>npm run build; tests.test_backend_api_persistence.BackendApiPersistenceTests.test_delete_active_order_removes_unscanned_order_and_queues_database_delete; tests.test_backend_api_persistence.BackendApiPersistenceTests.test_delete_active_order_idempotency_prevents_duplicate_audit_and_export; tests.test_backend_api_persistence.BackendApiPersistenceTests.test_delete_active_order_rejects_order_with_scans; tests.test_backend_telegram_import.BackendTelegramImportTests.test_telegram_worker_manual_delete_active_order_calls_safe_backend_endpoint; tests.test_backend_telegram_import.BackendTelegramImportTests.test_telegram_worker_manual_delete_refuses_started_order_before_backend_call</t>
         </is>
       </c>
     </row>
@@ -8067,17 +7751,17 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_backend_google_sheets_pending tests.test_google_sheets_sync_worker</t>
+          <t>python -m unittest tests.test_backend_db_only_runtime tests.test_google_sheets_decommission_contract</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Pending exports идемпотентны; batch scan/archive; rate limit ставит pause. Google-to-backend sync обновляет поля, но не удаляет backend item при пропаже строки и игнорирует ручной Google return marker без backend return.</t>
+          <t>Pending exports идемпотентны; batch scan/archive; rate limit ставит pause. database-to-backend sync обновляет поля, но не удаляет backend item при пропаже строки и игнорирует ручной backend return marker без backend return.</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Google pending export pauses on 429, keeps event pending with next_attempt_at, skips future retry events until cooldown, and continues newer ready events. Manual/live Google acceptance still pending.</t>
+          <t>database pending export pauses on 429, keeps event pending with next_attempt_at, skips future retry events until cooldown, and continues newer ready events. Manual/live database acceptance still pending.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -8088,7 +7772,7 @@
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>backend/app/google_sheets_pending.py; backend/app/google_sheets_sync_worker.py; tests/test_backend_google_sheets_pending.py; tests/test_google_sheets_sync_worker.py</t>
+          <t>backend/app/event_queue_service.py; backend/app/event_queue_service.py; tests/test_backend_db_only_runtime.py; tests/test_backend_db_only_runtime.py</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -8108,17 +7792,17 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>live Google Sheets credentials/quota</t>
+          <t>live PostgreSQL credentials/quota</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event OK; py_compile backend/app/google_sheets_pending.py tests/test_backend_google_sheets_pending.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event OK; py_compile backend/app/event_queue_service.py tests/test_backend_db_only_runtime.py OK.</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event</t>
+          <t>python -m unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event</t>
         </is>
       </c>
     </row>
@@ -8140,7 +7824,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Import строит dry-run; default mode dry_run, enabled ставит create events; unknown SKU/zero qty блокирует; already linked не дублируется; stock shortage может удалить unscanned active order и queued Google cleanup.</t>
+          <t>Import строит dry-run; default mode dry_run, enabled ставит create events; unknown SKU/zero qty блокирует; already linked не дублируется; stock shortage может удалить unscanned active order и queued database cleanup.</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -8208,7 +7892,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>DB source, Google mirror сравнивается по source keys, статусам/WH-R/dedup; Google down дает mirror_issue, не ломает DB workflow; критичные drift/SkladBot gaps создают incidents и Telegram notification events.</t>
+          <t>DB source, database state сравнивается по source keys, статусам/WH-R/dedup; database unavailable дает mirror_issue, не ломает DB workflow; критичные drift/SkladBot gaps создают incidents и Telegram notification events.</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -8254,7 +7938,7 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>tests.test_reconciliation_service.ReconciliationServiceTests.test_completed_item_in_active_multi_sku_order_matches_completed_google_row; tests.test_reconciliation_service.ReconciliationServiceTests.test_default_reconciliation_report_date_uses_business_timezone</t>
+          <t>tests.test_reconciliation_service.ReconciliationServiceTests.test_completed_item_in_active_multi_sku_order_matches_completed_database_row; tests.test_reconciliation_service.ReconciliationServiceTests.test_default_reconciliation_report_date_uses_business_timezone</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8028,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Compose поднимает Postgres, backend, frontend, SkladBot worker, Google sync worker, Telegram worker, Adminer behind Traefik. Backup/restore через pg_dump/psql; acceptance проверяет health/ready/compose/verifiers.</t>
+          <t>Compose поднимает Postgres, backend, frontend, SkladBot worker, database sync worker, Telegram worker, Adminer behind Traefik. Backup/restore через pg_dump/psql; acceptance проверяет health/ready/compose/verifiers.</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -8684,7 +8368,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Матчит по дате, клиенту, оплате, товарам/блокам; пишет found/multiple/not_found/pending; очередь Google export создается после обновления.</t>
+          <t>Матчит по дате, клиенту, оплате, товарам/блокам; пишет found/multiple/not_found/pending; очередь database event создается после обновления.</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -8956,7 +8640,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Postgres source of truth; сравнивает Google rows по source keys, статусы и WH-R; агрегирует SkladBot gaps; создает incidents и критичные Telegram alerts.</t>
+          <t>Postgres source of truth; сравнивает database rows по source keys, статусы и WH-R; агрегирует SkladBot gaps; создает incidents и критичные Telegram alerts.</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -8992,7 +8676,7 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>live Telegram bot/chat permissions; live Google Sheets credentials/quota; live SkladBot API/tokens</t>
+          <t>live Telegram bot/chat permissions; live PostgreSQL credentials/quota; live SkladBot API/tokens</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr">
@@ -9002,7 +8686,7 @@
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>tests.test_reconciliation_service.ReconciliationServiceTests.test_completed_item_in_active_multi_sku_order_matches_completed_google_row; tests.test_reconciliation_service.ReconciliationServiceTests.test_default_reconciliation_report_date_uses_business_timezone</t>
+          <t>tests.test_reconciliation_service.ReconciliationServiceTests.test_completed_item_in_active_multi_sku_order_matches_completed_database_row; tests.test_reconciliation_service.ReconciliationServiceTests.test_default_reconciliation_report_date_uses_business_timezone</t>
         </is>
       </c>
     </row>
@@ -9207,210 +8891,6 @@
       <c r="N45" s="2" t="inlineStr">
         <is>
           <t>python -m unittest tests.test_backend_api_persistence</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-001</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>auto+manual</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_backend_google_sheets_exporter</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Создает/обновляет layout, append/restore/delete rows, пишет сканы/status/SkladBot fields, переносит archive/cancel/no-KIZ/returns, сохраняет старый WH-R при pending.</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Python 3.12 temp venv: full unittest discover 509 tests OK; py_compile OK; 28/28 unique Test Loop unittest commands passed. Manual/live acceptance still pending.</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>manual_required</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr"/>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/google_sheets_exporter.py; tests/test_backend_google_sheets_exporter.py</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 13:31 Asia/Tashkent</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="M46" s="2" t="inlineStr">
-        <is>
-          <t>Full verifier: unittest discover 531 OK; py_compile OK; frontend build OK; compose/shell/audit/preflight/diff OK. Feature gate status OK but manual/open-error gates intentionally red.</t>
-        </is>
-      </c>
-      <c r="N46" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_backend_google_sheets_exporter</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-002</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>auto+manual</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_backend_google_sheets_pending</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>PendingEvent идемпотентен; scan/archive батчатся; PostgreSQL claim использует FOR UPDATE SKIP LOCKED; rate limit оставляет события pending с next_attempt_at; stale processing сбрасывается.</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>Targeted Google pending tests OK: PostgreSQL не использует session advisory lock и pending selection компилируется с FOR UPDATE SKIP LOCKED; rate limit leaves events pending. Manual Google/live quota acceptance still pending.</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>manual_required</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr"/>
-      <c r="H47" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/google_sheets_pending.py; tests/test_backend_google_sheets_pending.py</t>
-        </is>
-      </c>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 13:47 Asia/Tashkent</t>
-        </is>
-      </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L47" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="M47" s="2" t="inlineStr">
-        <is>
-          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_lock_does_not_use_session_level_advisory_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch - 3 tests OK</t>
-        </is>
-      </c>
-      <c r="N47" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_backend_google_sheets_pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-003</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>auto+manual</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_google_sheets_sync_worker</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Матчит по source IDs, обновляет поля, не затирает SkladBot stale mirror, импортирует КИЗы через movement checks, конфликты логирует вместо удаления DB truth.</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Python 3.12 temp venv: full unittest discover 509 tests OK; py_compile OK; 28/28 unique Test Loop unittest commands passed. Manual/live acceptance still pending.</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>manual_required</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr"/>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/google_sheets_sync_worker.py; tests/test_google_sheets_sync_worker.py</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 13:31 Asia/Tashkent</t>
-        </is>
-      </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="M48" s="2" t="inlineStr">
-        <is>
-          <t>Full verifier: unittest discover 531 OK; py_compile OK; frontend build OK; compose/shell/audit/preflight/diff OK. Feature gate status OK but manual/open-error gates intentionally red.</t>
-        </is>
-      </c>
-      <c r="N48" s="2" t="inlineStr">
-        <is>
-          <t>python -m unittest tests.test_google_sheets_sync_worker</t>
         </is>
       </c>
     </row>
@@ -9431,7 +8911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9786,7 +9266,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>src/taksklad/app_scanning.py; src/taksklad/scan_quantities.py; src/taksklad/desktop_scan_rules.py; tests/test_scan_quantities.py; tests/test_google_sheets_desktop_read.py; tests/test_desktop_ui_contract.py</t>
+          <t>src/taksklad/app_scanning.py; src/taksklad/scan_quantities.py; src/taksklad/desktop_scan_rules.py; tests/test_scan_quantities.py; tests/test_desktop_db_only_contract.py; tests/test_desktop_ui_contract.py</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -9937,12 +9417,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Локальный/pending откат сохраненного кода покрыт и исправлен: saved_codes_count теперь уменьшается без Google/backend. Откат уже синхронизированного кода без pending-записи всё ещё требует доступного backend или Google и ручной Windows validation.</t>
+          <t>Локальный/pending откат сохраненного кода покрыт и исправлен: saved_codes_count теперь уменьшается без database/backend. Откат уже синхронизированного кода без pending-записи всё ещё требует доступного backend или database и ручной Windows validation.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>src/taksklad/app_scanning.py; src/taksklad/pending_store.py; src/taksklad/backend_events.py; tests/test_desktop_pending_store.py; tests/test_desktop_ui_contract.py; tests/test_backend_bridge.py</t>
+          <t>src/taksklad/app_scanning.py; src/taksklad/pending_store.py; src/taksklad/backend_events.py; tests/test_desktop_db_only_contract.py; tests/test_desktop_ui_contract.py; tests/test_backend_bridge.py</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -9952,7 +9432,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Local/pending path fixed and covered. Validate live Windows undo for already-synced saved code with backend/Google available.</t>
+          <t>Local/pending path fixed and covered. Validate live Windows undo for already-synced saved code with backend/database available.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -10041,7 +9521,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Локальный риск очереди печати исправлен: finish/manual retry теперь проверяют успешную запись pending_print до печати и успешное удаление после печати до backend complete/Google archive. Физическая печать на Windows с реальным драйвером всё ещё требует validation.</t>
+          <t>Локальный риск очереди печати исправлен: finish/manual retry теперь проверяют успешную запись pending_print до печати и успешное удаление после печати до backend complete/backend completion. Физическая печать на Windows с реальным драйвером всё ещё требует validation.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -10145,12 +9625,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Локально исправлены unsupported extension UX, backend-mode preview дублей/invalid rows и потеря координат desktop parser -&gt; backend. Остается ручная validation: полный Tkinter e2e на Windows, live Yandex geocoder, backend/Google commit на тестовом файле и визуальный preview.</t>
+          <t>Локально исправлены unsupported extension UX, backend-mode preview дублей/invalid rows и потеря координат desktop parser -&gt; backend. Остается ручная validation: полный Tkinter e2e на Windows, live Yandex geocoder, backend/database commit на тестовом файле и визуальный preview.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/Google commit remain pending.</t>
+          <t>DESK-13 backend preview + coordinates regression: full unittest discover 558 tests OK; targeted import/parser/backend tests 27 OK; feature acceptance status OK; full py_compile OK; release_preflight --skip-network OK; git diff --check OK. Desktop backend import preview now calls /api/v1/imports/preview, filters duplicate/invalid rows before confirmation, and keeps coordinates in parsed records. Manual Windows Tkinter import, live geocoding, and real backend/database commit remain pending.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -10160,7 +9640,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Run manual Windows acceptance: choose .xlsx/.xlsm, verify preview counts for new/duplicate/invalid rows, confirm backend import, check active orders/logistics coordinates, legacy Google fallback, unsupported file warning, and live geocoding.</t>
+          <t>Run manual Windows acceptance: choose .xlsx/.xlsm, verify preview counts for new/duplicate/invalid rows, confirm backend import, check active orders/logistics coordinates, legacy legacy fallback, unsupported file warning, and live geocoding.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -10197,7 +9677,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Desktop return path подтвержден локально: confirmed_items отправляются в backend, backend-mode list/lookup не читает Google fallback, Google-only order без backend id отклоняется, legacy Google totals показывают реальные блоки/сумму.</t>
+          <t>Desktop return path подтвержден локально: confirmed_items отправляются в backend, backend-mode list/lookup не читает legacy fallback, legacy-only order без backend id отклоняется, legacy database totals показывают реальные блоки/сумму.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -10222,7 +9702,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_google_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects - 13 tests OK; python -m py_compile src/taksklad/app_returns.py tests/test_desktop_ui_contract.py backend/app/orders_service.py tests/test_backend_api_persistence.py - OK.</t>
+          <t>python -m unittest tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_totals_support_backend_and_legacy_item_shapes tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects - 13 tests OK; python -m py_compile src/taksklad/app_returns.py tests/test_desktop_ui_contract.py backend/app/orders_service.py tests/test_backend_api_persistence.py - OK.</t>
         </is>
       </c>
     </row>
@@ -10561,7 +10041,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Non-Postgres lock no-op в тестовой/локальной БД; ошибки Google не блокируют scan.</t>
+          <t>Non-Postgres lock no-op в тестовой/локальной БД; ошибки database не блокируют scan.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -10576,17 +10056,17 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Закрепить non-Postgres Google export lock контрактом и подтвердить, что Google export queue failure не блокирует scan API.</t>
+          <t>Закрепить non-Postgres database event lock контрактом и подтвердить, что database event queue failure не блокирует scan API.</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>tests/test_backend_google_sheets_pending.py</t>
+          <t>tests/test_backend_db_only_runtime.py</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_google_sheets_export_when_google_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_google_sheets_best_effort OK; py_compile backend/app/google_sheets_pending.py tests/test_backend_google_sheets_pending.py tests/test_backend_api_persistence.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_non_postgres_export_lock_returns_busy_without_processing tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_queues_database_export_when_database_is_down tests.test_backend_api_persistence.BackendApiPersistenceTests.test_scan_create_exports_scan_state_to_database_best_effort OK; py_compile backend/app/event_queue_service.py tests/test_backend_db_only_runtime.py tests/test_backend_api_persistence.py OK.</t>
         </is>
       </c>
     </row>
@@ -10613,7 +10093,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Backend return endpoint существует и является source of truth: Google mirror не переводит заказ в returned без backend; успешный возврат пишет movements, queues SkladBot return и Google exports.</t>
+          <t>Backend return endpoint существует и является source of truth: database state не переводит заказ в returned без backend; успешный возврат пишет movements, queues SkladBot return и database events.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -10628,7 +10108,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Закрепить backend source-of-truth return path targeted tests; Google остается best-effort mirror/export.</t>
+          <t>Закрепить backend source-of-truth return path targeted tests; database остается best-effort mirror/export.</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -10638,7 +10118,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_exports_archive_and_returns_to_google_sheets_best_effort tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_google_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_rejects_google_order_without_backend_id tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_uses_backend_id_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_legacy_return_keeps_google_write_fallback_for_google_order tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items - 12 tests OK</t>
+          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_lookup_and_mark_returned_excludes_order_from_active_list tests.test_backend_api_persistence.BackendApiPersistenceTests.test_return_releases_kiz_for_new_outbound_scan_with_history tests.test_backend_api_persistence.BackendApiPersistenceTests.test_failed_return_does_not_release_kiz_for_new_order tests.test_backend_api_persistence tests.test_backend_api_persistence.BackendApiPersistenceTests.test_mark_return_rejects_mismatched_confirmed_items_without_side_effects tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_mark_sends_confirmed_items_to_backend tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_returns_list_reads_backend_without_database_fallback tests.test_desktop_ui_contract.DesktopUiContractTests.test_backend_return_lookup_reads_backend_without_database_fallback tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_db_only_contract tests.test_desktop_ui_contract.DesktopUiContractTests.test_return_confirmed_items_are_built_from_backend_items - 12 tests OK</t>
         </is>
       </c>
     </row>
@@ -10665,7 +10145,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Google export failure не откатывает Postgres; частичные ошибки требуют incident review.</t>
+          <t>database event failure не откатывает Postgres; частичные ошибки требуют incident review.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -10680,7 +10160,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Сделать backend import независимым от post-commit Google export queue failure и записывать incident/audit для operator review.</t>
+          <t>Сделать backend import независимым от post-commit database event queue failure и записывать incident/audit для operator review.</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -10690,7 +10170,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_google_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_google_sheets_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_google_sheets tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write OK; py_compile backend/app/imports_service.py tests/test_backend_api_persistence.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_reports_database_queue_failure_without_rolling_back_backend_data tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_keeps_backend_data_when_database_export_fails tests.test_backend_api_persistence.BackendApiPersistenceTests.test_duplicate_backend_import_still_can_backfill_database tests.test_backend_api_persistence.BackendApiPersistenceTests.test_import_preview_reports_duplicates_invalid_rows_and_does_not_write OK; py_compile backend/app/imports_service.py tests/test_backend_api_persistence.py OK.</t>
         </is>
       </c>
     </row>
@@ -10925,12 +10405,12 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Google quota/429 останавливает batch до retry; mirror drift требует reconciliation.</t>
+          <t>database availability/429 останавливает batch до retry; mirror drift требует reconciliation.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>backend/app/google_sheets_pending.py; backend/app/google_sheets_sync_worker.py; tests/test_backend_google_sheets_pending.py; tests/test_google_sheets_sync_worker.py</t>
+          <t>backend/app/event_queue_service.py; backend/app/event_queue_service.py; tests/test_backend_db_only_runtime.py; tests/test_backend_db_only_runtime.py</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -10940,17 +10420,17 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Уважать payload.next_attempt_at после Google 429/quota и не блокировать готовые более новые pending exports.</t>
+          <t>Уважать payload.next_attempt_at после database 429/quota и не блокировать готовые более новые pending exports.</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>backend/app/google_sheets_pending.py; tests/test_backend_google_sheets_pending.py</t>
+          <t>backend/app/event_queue_service.py; tests/test_backend_db_only_runtime.py</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Targeted verifier: unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event OK; py_compile backend/app/google_sheets_pending.py tests/test_backend_google_sheets_pending.py OK.</t>
+          <t>Targeted verifier: unittest tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_future_retry_after_event_does_not_block_newer_ready_event tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_db_only_runtime.databaseSheetsPendingLockTests.test_bad_event_does_not_block_newer_valid_event OK; py_compile backend/app/event_queue_service.py tests/test_backend_db_only_runtime.py OK.</t>
         </is>
       </c>
     </row>
@@ -11029,7 +10509,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Returned DB status может легитимно соответствовать Google Выполнено; риск регрессии высокий.</t>
+          <t>Returned DB status может легитимно соответствовать database Выполнено; риск регрессии высокий.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -11044,7 +10524,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Returned-vs-Google status and active multi-SKU completed item reconciliation regressions are covered locally.</t>
+          <t>Returned-vs-database status and active multi-SKU completed item reconciliation regressions are covered locally.</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -11601,7 +11081,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>API endpoint сам не шлет alerts; при недоступном Google статус mirror_issue без деталей mismatch.</t>
+          <t>API endpoint сам не шлет alerts; при недоступном database статус mirror_issue без деталей mismatch.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -11789,188 +11269,188 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>GAP-045</t>
+          <t>ERR-001</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>TS-GS-001</t>
+          <t>PG-01; OPS-01</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>risk_or_test_gap</t>
+          <t>test_environment</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>При credentials выполняет реальные Google writes; без них действия должны ретраиться через очередь.</t>
+          <t>Project .venv rebuilt to Python 3.12.13 with desktop and backend requirements; backend tests no longer require temporary /tmp venv.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>backend/app/google_sheets_exporter.py; tests/test_backend_google_sheets_exporter.py</t>
+          <t>docs/local-development-setup.md; requirements.txt; backend/requirements.txt</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>accepted</t>
+          <t>fixed_retested</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+          <t>Rebuild .venv with python3.12 and install requirements.txt + backend/requirements.txt; keep old Python 3.9 venv as local backup.</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>production smoke 2026-07-02</t>
+          <t>local .venv rebuild; docs/local-development-setup.md</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
+          <t>.venv/bin/python --version = Python 3.12.13; .venv/bin/python -m unittest discover -s tests = 531 tests OK; .venv/bin/python -m py_compile ... = OK; backup archive/local-venv-backups/.venv.py39-backup-20260622T1408 kept</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>GAP-046</t>
+          <t>ERR-002</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>TS-GS-002</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>risk_or_test_gap</t>
+          <t>test_register_quality</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>PostgreSQL Google export queue intentionally does not use session-level advisory lock; pending selection uses FOR UPDATE SKIP LOCKED row locking and stale processing reset.</t>
+          <t>Initial spreadsheet used pytest-style commands while project runbook uses unittest and pytest is not a declared dependency.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>backend/app/google_sheets_pending.py; tests/test_backend_google_sheets_pending.py; docs/event-queue-lifecycle.md</t>
+          <t>docs/taksklad-feature-user-stories.xlsx Test Loop commands</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>fixed_retested</t>
+          <t>fixed</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Keep PostgreSQL session advisory lock disabled to avoid pooled-connection busy state; assert row-level FOR UPDATE SKIP LOCKED contract in tests.</t>
+          <t>Converted spreadsheet test commands to unittest module commands and separated automated/manual status columns.</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>tests/test_backend_google_sheets_pending.py; docs/event-queue-lifecycle.md</t>
+          <t>docs/taksklad-feature-user-stories.xlsx</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>/tmp/taksklad-test-py312/bin/python -m unittest tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_lock_does_not_use_session_level_advisory_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_postgres_pending_selection_uses_skip_locked_row_lock tests.test_backend_google_sheets_pending.GoogleSheetsPendingLockTests.test_rate_limit_keeps_event_pending_and_stops_batch - 3 tests OK</t>
+          <t>Retest with generated unittest command list in this loop.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>GAP-047</t>
+          <t>ERR-003</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>TS-GS-003</t>
+          <t>OPS-01</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>risk_or_test_gap</t>
+          <t>test_register_quality</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>High-risk режим: Google может писать в Postgres; manual return columns игнорируются без backend return source.</t>
+          <t>OPS-01 test command mixed local unittest and live VDS acceptance in one shell-like string.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>backend/app/google_sheets_sync_worker.py; tests/test_google_sheets_sync_worker.py</t>
+          <t>docs/taksklad-feature-user-stories.xlsx</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>accepted</t>
+          <t>fixed</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Closed by production smoke acceptance and live readiness checks for this stage.</t>
+          <t>Separated local unittest command from VDS manual acceptance note.</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>production smoke 2026-07-02</t>
+          <t>docs/taksklad-feature-user-stories.xlsx</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>Stage acceptance closed by operator production smoke plus live public readiness checks. Not individually replayed by Codex on warehouse Windows hardware.</t>
+          <t>Pending local retest in current loop; VDS acceptance still manual/live.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>ERR-001</t>
+          <t>ERR-004</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>PG-01; OPS-01</t>
+          <t>API-10; TS-REC-001</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>test_environment</t>
+          <t>logistics_bug</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Project .venv rebuilt to Python 3.12.13 with desktop and backend requirements; backend tests no longer require temporary /tmp venv.</t>
+          <t>Daily reconciliation reported false action_required for active multi-SKU order with one completed item mirrored in database as Выполнено.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>docs/local-development-setup.md; requirements.txt; backend/requirements.txt</t>
+          <t>backend/app/reconciliation_service.py; tests/test_reconciliation_service.py</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -11980,379 +11460,223 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Rebuild .venv with python3.12 and install requirements.txt + backend/requirements.txt; keep old Python 3.9 venv as local backup.</t>
+          <t>Compare database status against item-level sheet status while preserving returned order compatibility.</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>local .venv rebuild; docs/local-development-setup.md</t>
+          <t>backend/app/reconciliation_service.py; tests/test_reconciliation_service.py</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>.venv/bin/python --version = Python 3.12.13; .venv/bin/python -m unittest discover -s tests = 531 tests OK; .venv/bin/python -m py_compile ... = OK; backup archive/local-venv-backups/.venv.py39-backup-20260622T1408 kept</t>
+          <t>Regression selector OK; full unittest discover 526 OK; py_compile OK. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>ERR-002</t>
+          <t>ERR-005</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>DESK-04</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>test_register_quality</t>
+          <t>ux_bug</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Initial spreadsheet used pytest-style commands while project runbook uses unittest and pytest is not a declared dependency.</t>
+          <t>Order-list search card showed only matching SKU summary for a multi-SKU order, understating total SKU/blocks.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>docs/taksklad-feature-user-stories.xlsx Test Loop commands</t>
+          <t>src/taksklad/order_list_models.py; tests/test_order_list_models.py</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>fixed_retested</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Converted spreadsheet test commands to unittest module commands and separated automated/manual status columns.</t>
+          <t>Build visible card summary from full grouped order, not filtered search subset.</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>docs/taksklad-feature-user-stories.xlsx</t>
+          <t>src/taksklad/order_list_models.py; tests/test_order_list_models.py</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>Retest with generated unittest command list in this loop.</t>
+          <t>Regression selector OK; full unittest discover 526 OK; py_compile OK. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>ERR-003</t>
+          <t>ERR-006</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>API-10; TS-REC-001</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
+          <t>logistics_bug</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Reconciliation without report_date defaulted to UTC date instead of warehouse business date Asia/Tashkent.</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>backend/app/reconciliation_service.py; tests/test_reconciliation_service.py</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>fixed_retested</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Use report_timezone() for default reconciliation report date.</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>backend/app/reconciliation_service.py; tests/test_reconciliation_service.py</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>Regression selector OK; full unittest discover 526 OK; py_compile OK. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ERR-007</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
           <t>test_register_quality</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>OPS-01 test command mixed local unittest and live VDS acceptance in one shell-like string.</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>docs/taksklad-feature-user-stories.xlsx</t>
-        </is>
-      </c>
-      <c r="G51" s="2" t="inlineStr">
-        <is>
-          <t>fixed</t>
-        </is>
-      </c>
-      <c r="H51" s="2" t="inlineStr">
-        <is>
-          <t>Separated local unittest command from VDS manual acceptance note.</t>
-        </is>
-      </c>
-      <c r="I51" s="2" t="inlineStr">
-        <is>
-          <t>docs/taksklad-feature-user-stories.xlsx</t>
-        </is>
-      </c>
-      <c r="J51" s="2" t="inlineStr">
-        <is>
-          <t>Pending local retest in current loop; VDS acceptance still manual/live.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>ERR-004</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>API-10; TS-REC-001</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>logistics_bug</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>Daily reconciliation reported false action_required for active multi-SKU order with one completed item mirrored in Google as Выполнено.</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/reconciliation_service.py; tests/test_reconciliation_service.py</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Feature user stories spreadsheet had no automated guard for schema drift, duplicate Feature IDs, stale pytest commands or missing evidence files.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>docs/taksklad-feature-user-stories.xlsx; tests/test_feature_user_stories_register.py</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
         <is>
           <t>fixed_retested</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t>Compare Google status against item-level sheet status while preserving returned order compatibility.</t>
-        </is>
-      </c>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/reconciliation_service.py; tests/test_reconciliation_service.py</t>
-        </is>
-      </c>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>Regression selector OK; full unittest discover 526 OK; py_compile OK. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Added workbook structure/register validator test and updated status validation vocabulary.</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>tests/test_feature_user_stories_register.py; docs/taksklad-feature-user-stories.xlsx</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>tests.test_feature_user_stories_register - 4 tests OK; full unittest discover 526 OK. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>ERR-005</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>DESK-04</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>ux_bug</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ERR-008</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>test_register_quality</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>Order-list search card showed only matching SKU summary for a multi-SKU order, understating total SKU/blocks.</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>src/taksklad/order_list_models.py; tests/test_order_list_models.py</t>
-        </is>
-      </c>
-      <c r="G53" s="2" t="inlineStr">
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Feature register had no CLI gate to block completion while Manual Acceptance rows, missing manual rows, unknown statuses or Errors rows remained open.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>docs/taksklad-feature-user-stories.xlsx; tools/feature_acceptance_status.py; tests/test_feature_acceptance_status.py</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
         <is>
           <t>fixed_retested</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
-        <is>
-          <t>Build visible card summary from full grouped order, not filtered search subset.</t>
-        </is>
-      </c>
-      <c r="I53" s="2" t="inlineStr">
-        <is>
-          <t>src/taksklad/order_list_models.py; tests/test_order_list_models.py</t>
-        </is>
-      </c>
-      <c r="J53" s="2" t="inlineStr">
-        <is>
-          <t>Regression selector OK; full unittest discover 526 OK; py_compile OK. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>ERR-006</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>API-10; TS-REC-001</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>logistics_bug</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>Reconciliation without report_date defaulted to UTC date instead of warehouse business date Asia/Tashkent.</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/reconciliation_service.py; tests/test_reconciliation_service.py</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>fixed_retested</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr">
-        <is>
-          <t>Use report_timezone() for default reconciliation report date.</t>
-        </is>
-      </c>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/reconciliation_service.py; tests/test_reconciliation_service.py</t>
-        </is>
-      </c>
-      <c r="J54" s="2" t="inlineStr">
-        <is>
-          <t>Regression selector OK; full unittest discover 526 OK; py_compile OK. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>ERR-007</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>test_register_quality</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Feature user stories spreadsheet had no automated guard for schema drift, duplicate Feature IDs, stale pytest commands or missing evidence files.</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>docs/taksklad-feature-user-stories.xlsx; tests/test_feature_user_stories_register.py</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>fixed_retested</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>Added workbook structure/register validator test and updated status validation vocabulary.</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>tests/test_feature_user_stories_register.py; docs/taksklad-feature-user-stories.xlsx</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>tests.test_feature_user_stories_register - 4 tests OK; full unittest discover 526 OK. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>ERR-008</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>test_register_quality</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Feature register had no CLI gate to block completion while Manual Acceptance rows, missing manual rows, unknown statuses or Errors rows remained open.</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>docs/taksklad-feature-user-stories.xlsx; tools/feature_acceptance_status.py; tests/test_feature_acceptance_status.py</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>fixed_retested</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
+      <c r="H53" t="inlineStr">
         <is>
           <t>Added feature_acceptance_status.py with JSON summary and --require-manual-complete / --require-no-open-errors exit gates.</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>tools/feature_acceptance_status.py; tests/test_feature_acceptance_status.py; docs/taksklad-feature-user-stories.xlsx</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="J53" t="inlineStr">
         <is>
           <t>tests.test_feature_acceptance_status tests.test_feature_user_stories_register - 14 tests OK; full unittest discover 526 OK; manual gate exits 3; open-errors gate exits 4. Full unittest discover 531 OK; py_compile/build/preflight/diff OK.</t>
         </is>
@@ -12419,7 +11743,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Excel import, KIZ scan, Google Sheets, Telegram, SkladBot, reports, auto-update</t>
+          <t>Excel import, KIZ scan, PostgreSQL, Telegram, SkladBot, reports, auto-update</t>
         </is>
       </c>
     </row>
@@ -12612,7 +11936,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Telegram/SkladBot/Google/reports extraction</t>
+          <t>Telegram/SkladBot/database/reports extraction</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -12699,7 +12023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12794,7 +12118,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Entry points вызывают run_app; --smoke-import проверяет импорт; без Google credentials и без backend-read показывается startup error.</t>
+          <t>Entry points вызывают run_app; --smoke-import проверяет импорт; без database credentials и без backend-read показывается startup error.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -12898,7 +12222,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Backend read mode использует backend как primary; при падении backend идет Google fallback; SkladBot error не скрывает Google-заказы; текущая позиция сохраняется при refresh.</t>
+          <t>Backend read mode использует backend как primary; при падении backend идет legacy fallback; SkladBot error не скрывает database-заказы; текущая позиция сохраняется при refresh.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -13210,7 +12534,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Undo пишет backup, обновляет pending save/backend/Google, может очистить active row через allow_empty=True, блокирует finish если позиция стала неполной; archive/return/closed не откатывает.</t>
+          <t>Undo пишет backup, обновляет pending save/backend/database, может очистить active row через allow_empty=True, блокирует finish если позиция стала неполной; archive/return/closed не откатывает.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -13262,7 +12586,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>next_product требует exact plan, сохраняет в backend или Google, retryable Google error кладет pending save, пишет backup, последняя позиция ведет к ЗАВЕРШИТЬ ЗАКАЗ.</t>
+          <t>next_product требует exact plan, сохраняет в backend или database, retryable database error кладет pending save, пишет backup, последняя позиция ведет к ЗАВЕРШИТЬ ЗАКАЗ.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -13314,7 +12638,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Finish требует все позиции saved/full scanned; подтверждает параметры печати; add_pending_print создается до печати; backend complete/Google archive только после успешной печати.</t>
+          <t>Finish требует все позиции saved/full scanned; подтверждает параметры печати; add_pending_print создается до печати; backend complete/backend completion только после успешной печати.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -13470,7 +12794,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Окно ищет заявку, показывает состав, требует подтверждение items; backend mode читает/пишет backend; Google-only возврат без _backend_order_id в backend mode отклоняется; legacy Google fallback сохранен.</t>
+          <t>Окно ищет заявку, показывает состав, требует подтверждение items; backend mode читает/пишет backend; legacy-only возврат без _backend_order_id в backend mode отклоняется; legacy legacy fallback сохранен.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -13730,7 +13054,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/admin/table строит плоские строки по позициям, totals по всем строкам, recent audit, pending Google count; UI фильтрует по дате, статусу, сканам, SkladBot, Google.</t>
+          <t>/api/v1/admin/table строит плоские строки по позициям, totals по всем строкам, recent audit, pending database count; UI фильтрует по дате, статусу, сканам, SkladBot, database.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -13782,7 +13106,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Scan валидирует код, блокирует КИЗ PostgreSQL advisory lock, проверяет дубль/другой заказ/SKU/aggregate box, пишет scan_codes, kiz_movements, audit и очередь Google export. Undo пишет movement undo, удаляет scan, пересчитывает blocks.</t>
+          <t>Scan валидирует код, блокирует КИЗ PostgreSQL advisory lock, проверяет дубль/другой заказ/SKU/aggregate box, пишет scan_codes, kiz_movements, audit и очередь database event. Undo пишет movement undo, удаляет scan, пересчитывает blocks.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -13834,7 +13158,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Complete требует все required blocks и повторный complete идемпотентен. Return ищет completed order, требует подтверждение всех позиций, пишет return movement, очередь SkladBot return и Google archive/returns exports.</t>
+          <t>Complete требует все required blocks и повторный complete идемпотентен. Return ищет completed order, требует подтверждение всех позиций, пишет return movement, очередь SkladBot return и backend completion/returns exports.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -13886,7 +13210,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/imports создает ImportJob, группирует orders/items, дедупит по source/import keys, backfill адресов, создает incident при ошибках, ставит Google import export и SkladBot dry-run.</t>
+          <t>/api/v1/imports создает ImportJob, группирует orders/items, дедупит по source/import keys, backfill адресов, создает incident при ошибках, ставит database import export и SkladBot dry-run.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -13938,7 +13262,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>UI требует выбор, reason, confirm, expected updated_at; backend повторно проверяет активность, сканы, pending Google, idempotency, audit и queue exports.</t>
+          <t>UI требует выбор, reason, confirm, expected updated_at; backend повторно проверяет активность, сканы, pending database, idempotency, audit и queue exports.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -14126,27 +13450,27 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Backend / Google</t>
+          <t>Backend / Database</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Google mirror sync/pending</t>
+          <t>DB-only runtime and XLSX interchange</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>live Google Sheets credentials/quota</t>
+          <t>live PostgreSQL credentials/quota</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Run against configured Google Sheets mirror with safe test order and verify pending/export/sync result.</t>
+          <t>Run against configured PostgreSQL mirror with safe test order and verify pending/export/sync result.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Pending exports идемпотентны; batch scan/archive; rate limit ставит pause. Google-to-backend sync обновляет поля, но не удаляет backend item при пропаже строки и игнорирует ручной Google return marker без backend return.</t>
+          <t>Pending exports идемпотентны; batch scan/archive; rate limit ставит pause. database-to-backend sync обновляет поля, но не удаляет backend item при пропаже строки и игнорирует ручной backend return marker без backend return.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -14198,7 +13522,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Import строит dry-run; default mode dry_run, enabled ставит create events; unknown SKU/zero qty блокирует; already linked не дублируется; stock shortage может удалить unscanned active order и queued Google cleanup.</t>
+          <t>Import строит dry-run; default mode dry_run, enabled ставит create events; unknown SKU/zero qty блокирует; already linked не дублируется; stock shortage может удалить unscanned active order и queued database cleanup.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -14250,7 +13574,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>DB source, Google mirror сравнивается по source keys, статусам/WH-R/dedup; Google down дает mirror_issue, не ломает DB workflow; критичные drift/SkladBot gaps создают incidents и Telegram notification events.</t>
+          <t>DB source, database state сравнивается по source keys, статусам/WH-R/dedup; database unavailable дает mirror_issue, не ломает DB workflow; критичные drift/SkladBot gaps создают incidents и Telegram notification events.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -14354,7 +13678,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Compose поднимает Postgres, backend, frontend, SkladBot worker, Google sync worker, Telegram worker, Adminer behind Traefik. Backup/restore через pg_dump/psql; acceptance проверяет health/ready/compose/verifiers.</t>
+          <t>Compose поднимает Postgres, backend, frontend, SkladBot worker, database sync worker, Telegram worker, Adminer behind Traefik. Backup/restore через pg_dump/psql; acceptance проверяет health/ready/compose/verifiers.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -14614,7 +13938,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Матчит по дате, клиенту, оплате, товарам/блокам; пишет found/multiple/not_found/pending; очередь Google export создается после обновления.</t>
+          <t>Матчит по дате, клиенту, оплате, товарам/блокам; пишет found/multiple/not_found/pending; очередь database event создается после обновления.</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -14807,12 +14131,12 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Postgres vs Google/SkladBot</t>
+          <t>Postgres vs database/SkladBot</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>live Telegram bot/chat permissions; live Google Sheets credentials/quota; live SkladBot API/tokens</t>
+          <t>live Telegram bot/chat permissions; live PostgreSQL credentials/quota; live SkladBot API/tokens</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -14822,7 +14146,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Postgres source of truth; сравнивает Google rows по source keys, статусы и WH-R; агрегирует SkladBot gaps; создает incidents и критичные Telegram alerts.</t>
+          <t>Postgres source of truth; сравнивает database rows по source keys, статусы и WH-R; агрегирует SkladBot gaps; создает incidents и критичные Telegram alerts.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -14945,162 +14269,6 @@
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-02 16:52 Asia/Tashkent</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-001</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Google Sheets</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Backend-to-Google exporter</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>Run against configured Google Sheets mirror with safe test order and verify pending/export/sync result.</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>Создает/обновляет layout, append/restore/delete rows, пишет сканы/status/SkladBot fields, переносит archive/cancel/no-KIZ/returns, сохраняет старый WH-R при pending.</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>accepted</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
-        </is>
-      </c>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
-        </is>
-      </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-02 16:52 Asia/Tashkent</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-002</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>Google Sheets</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Pending export retry</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>Run against configured Google Sheets mirror with safe test order and verify pending/export/sync result.</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>PendingEvent идемпотентен; scan/archive батчатся; rate limit оставляет события pending с next_attempt_at; stale processing сбрасывается.</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>accepted</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
-        </is>
-      </c>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
-        </is>
-      </c>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-02 16:52 Asia/Tashkent</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>TS-GS-003</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Google Sheets</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Google-to-backend sync</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>live Google Sheets credentials/quota</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Run against configured Google Sheets mirror with safe test order and verify pending/export/sync result.</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Матчит по source IDs, обновляет поля, не затирает SkladBot stale mirror, импортирует КИЗы через movement checks, конфликты логирует вместо удаления DB truth.</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>accepted</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>Accepted by Anton production smoke on 2026-07-02: Smartup auto export, Telegram imports into DB, KIZ scanning, and SkladBot request creation worked in live flow; no operator-visible errors reported. Codex live checks: /health ok, /ready ok, DB/migrations ok, queue last_errors empty and stale_processing_count=0.</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>User production smoke confirmation 2026-07-02; outputs/taksklad_acceptance/ACCEPTANCE_RESULTS.md; curl https://api.taksklad.uz/health; curl https://api.taksklad.uz/ready; GitHub Actions CI/Deploy green on main.</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
         <is>
           <t>2026-07-02 16:52 Asia/Tashkent</t>
         </is>

</xml_diff>